<commit_message>
🔄 Auto-collect traffic data: 2026-09-21 10:13 AM IST
</commit_message>
<xml_diff>
--- a/output/excel/Bus_vs_Metro_Data_2026-09-21_Mon.xlsx
+++ b/output/excel/Bus_vs_Metro_Data_2026-09-21_Mon.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="All Periods Combined" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="All Periods Combined" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1162" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2208" uniqueCount="536">
   <si>
     <t>Date</t>
   </si>
@@ -140,7 +141,7 @@
     <t>12:00 AM</t>
   </si>
   <si>
-    <t>Sunday (Weekend) - Night Off-Peak</t>
+    <t>Monday (Weekday) - Night Off-Peak</t>
   </si>
   <si>
     <t>Bus</t>
@@ -950,6 +951,594 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/12_00_AM/MC-25/car.jpg</t>
   </si>
   <si>
+    <t>9/21/2026, 10:02:32 AM</t>
+  </si>
+  <si>
+    <t>10:00 AM</t>
+  </si>
+  <si>
+    <t>Monday (Weekday) - Morning Peak</t>
+  </si>
+  <si>
+    <t> | 50 min | 10:00 AM—10:50 AM | DN-9/1  234/1 | 10:00 AM from Dakshineswar | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 10:00 AM—10:28 AM | Blue Line | 10:00 AM from Dakshineswar | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-01/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-01/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:02:59 AM</t>
+  </si>
+  <si>
+    <t> | 51 min | 10:04 AM—10:55 AM | S-112 | 10:04 AM from Khudiram Metro | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 10:03 AM—10:31 AM | Blue Line | 10:03 AM from Shahid Khudiram | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-02/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-02/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:03:26 AM</t>
+  </si>
+  <si>
+    <t>S-168</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:07 AM—10:19 AM | S-168 | 10:07 AM from Dumdum Station | Details</t>
+  </si>
+  <si>
+    <t> | 7 min | 10:05 AM—10:12 AM | Blue Line | 10:05 AM from Shyambazar | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>1.71x</t>
+  </si>
+  <si>
+    <t>41.7% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-03/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-03/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:03:53 AM</t>
+  </si>
+  <si>
+    <t>S-10</t>
+  </si>
+  <si>
+    <t> | 18 min | 10:05 AM—10:23 AM | S-10 | 10:05 AM from Shyambazar | Details</t>
+  </si>
+  <si>
+    <t> | 11 min | 10:05 AM—10:16 AM | Blue Line | 10:05 AM from Shyambazar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-04/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-04/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:04:20 AM</t>
+  </si>
+  <si>
+    <t> | 18 min | 10:04 AM—10:22 AM | 40A | 10:04 AM from S.P. Mukherjee Road / R.B. Avenue Crossing | Details</t>
+  </si>
+  <si>
+    <t> | 11 min | 10:02 AM—10:13 AM | Blue Line | 10:02 AM from Kalighat | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-05/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-05/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:04:48 AM</t>
+  </si>
+  <si>
+    <t> | 24 min | 10:00 AM—10:24 AM | DN-9/1 | 10:00 AM from Dakshineswar | Details</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:00 AM—10:12 AM | Blue Line | 10:00 AM from Dakshineswar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-06/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:05:16 AM</t>
+  </si>
+  <si>
+    <t> | 27 min | 10:11 AM—10:38 AM | 12C/1B | 10:11 AM from Esplanade Metro | Details</t>
+  </si>
+  <si>
+    <t> | 17 min | 10:04 AM—10:21 AM | Blue Line | 10:04 AM from Esplanade | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>1.59x</t>
+  </si>
+  <si>
+    <t>37.0% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-07/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-07/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:05:42 AM</t>
+  </si>
+  <si>
+    <t> | 22 min | 10:09 AM—10:31 AM | S-112 | 10:09 AM from Tollygunge Tram Depot | Details</t>
+  </si>
+  <si>
+    <t> | 15 min | 10:03 AM—10:18 AM | Blue Line | 10:03 AM from Mahanayak Uttam Kumar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-08/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-08/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:06:09 AM</t>
+  </si>
+  <si>
+    <t> | 36 min | 10:00 AM—10:36 AM | 30B   | 10:00 AM from Dumdum Station |  3 min | Details</t>
+  </si>
+  <si>
+    <t> | 16 min | 10:00 AM—10:16 AM | Blue Line | 10:00 AM from Dumdum | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-09/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-09/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:06:37 AM</t>
+  </si>
+  <si>
+    <t> | 40 min | 10:00 AM—10:40 AM | 215A/1 | 10:00 AM from Howrah Station | Details</t>
+  </si>
+  <si>
+    <t> | 30 min | 10:02 AM—10:32 AM | Green Line | 10:02 AM from Howrah | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t>25.0% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-10/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-10/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:07:04 AM</t>
+  </si>
+  <si>
+    <t>S-12</t>
+  </si>
+  <si>
+    <t> | 26 min | 10:02 AM—10:28 AM | S-12 | 10:02 AM from Sealdah - B.R. Singh Hospital | Details</t>
+  </si>
+  <si>
+    <t> | 21 min | 10:05 AM—10:26 AM | Green Line | 10:05 AM from Sealdah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>1.24x</t>
+  </si>
+  <si>
+    <t>19.2% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-11/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-11/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:07:31 AM</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>Walk &gt; Bus Walk</t>
+  </si>
+  <si>
+    <t> | 27 min | 10:00 AM—10:27 AM |   72 </t>
+  </si>
+  <si>
+    <t> | 11 min | 10:00 AM—10:11 AM | Green Line | 10:00 AM from Howrah Maidan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>2.45x</t>
+  </si>
+  <si>
+    <t>59.3% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-12/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-12/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:07:58 AM</t>
+  </si>
+  <si>
+    <t> | 26 min | 10:02 AM—10:28 AM | S-21  S-12 | 10:02 AM from Phoolbagan | Details</t>
+  </si>
+  <si>
+    <t> | 18 min | 10:02 AM—10:20 AM | Green Line | 10:02 AM from Phoolbagan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>8 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.44x</t>
+  </si>
+  <si>
+    <t>30.8% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-13/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-13/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:08:26 AM</t>
+  </si>
+  <si>
+    <t> | 29 min | 10:00 AM—10:29 AM | 44/1 | 10:00 AM from Howrah Station |  2 min | Details</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:02 AM—10:14 AM | Green Line | 10:02 AM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>17 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.42x</t>
+  </si>
+  <si>
+    <t>58.6% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-14/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-14/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:08:54 AM</t>
+  </si>
+  <si>
+    <t> | 34 min | 10:20 AM—10:54 AM | S-12N | 10:20 AM from Esplanade Metro | Details</t>
+  </si>
+  <si>
+    <t> | 25 min | 10:01 AM—10:26 AM | Green Line | 10:01 AM from Esplanade | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t>26.5% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-15/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-15/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:09:20 AM</t>
+  </si>
+  <si>
+    <t>AS-3</t>
+  </si>
+  <si>
+    <t> | 36 min | 10:03 AM—10:39 AM | AS-3 | 10:03 AM from Dhalai Bridge | Details</t>
+  </si>
+  <si>
+    <t>Orange Line</t>
+  </si>
+  <si>
+    <t> | 23 min | 10:20 AM—10:43 AM | Orange Line | 10:20 AM from Kavi Subhash | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>13 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.57x</t>
+  </si>
+  <si>
+    <t>36.1% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-16/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-16/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:09:47 AM</t>
+  </si>
+  <si>
+    <t> | 16 min | 10:00 AM—10:16 AM | V-1 | 10:00 AM from Ruby | Details</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:06 AM—10:18 AM | Orange Line | 10:06 AM from Hemanta Mukhopadhyay | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>4 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-17/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-17/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:10:14 AM</t>
+  </si>
+  <si>
+    <t>C26A</t>
+  </si>
+  <si>
+    <t> | 47 min | 10:02 AM—10:49 AM |   C26A</t>
+  </si>
+  <si>
+    <t> | 19 min | 10:20 AM—10:39 AM | Orange Line | 10:20 AM from Kavi Subhash | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>28 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.47x</t>
+  </si>
+  <si>
+    <t>59.6% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-18/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-18/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:10:40 AM</t>
+  </si>
+  <si>
+    <t> | 26 min | 10:01 AM—10:27 AM | S-131 | 10:01 AM from Diamond Park | Details</t>
+  </si>
+  <si>
+    <t>Purple Line</t>
+  </si>
+  <si>
+    <t> | 17 min | 10:14 AM—10:31 AM | Purple Line | 10:14 AM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>1.53x</t>
+  </si>
+  <si>
+    <t>34.6% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-19/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-19/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:11:07 AM</t>
+  </si>
+  <si>
+    <t>222</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:01 AM—10:13 AM | 222 | 10:01 AM from Behala Chowrasta | Details</t>
+  </si>
+  <si>
+    <t> | 9 min | 10:01 AM—10:10 AM | Purple Line | 10:01 AM from Behala Chowrasta | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-20/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-20/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:11:34 AM</t>
+  </si>
+  <si>
+    <t> | 14 min | 10:01 AM—10:15 AM | S-131 | 10:01 AM from Diamond Park | Details</t>
+  </si>
+  <si>
+    <t> | 8 min | 10:14 AM—10:22 AM | Purple Line | 10:14 AM from Joka | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>6 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.75x</t>
+  </si>
+  <si>
+    <t>42.9% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-21/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-21/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:12:01 AM</t>
+  </si>
+  <si>
+    <t> | 22 min | 10:01 AM—10:23 AM | S-131 | 10:01 AM from Diamond Park | Details</t>
+  </si>
+  <si>
+    <t> | 14 min | 10:14 AM—10:28 AM | Purple Line | 10:14 AM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>36.4% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-22/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-22/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:12:27 AM</t>
+  </si>
+  <si>
+    <t> | 8 min | 10:01 AM—10:09 AM | 222 | 10:01 AM from Behala Chowrasta | Details</t>
+  </si>
+  <si>
+    <t> | 6 min | 10:01 AM—10:07 AM | Purple Line | 10:01 AM from Behala Chowrasta | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>2 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-23/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-23/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:12:55 AM</t>
+  </si>
+  <si>
+    <t> | 4 min | 10:01 AM—10:05 AM | S-3B | 10:01 AM from Pathak Para | Details</t>
+  </si>
+  <si>
+    <t> | 3 min | 10:07 AM—10:10 AM | Purple Line | 10:07 AM from Taratala | ₹5.00 | Details</t>
+  </si>
+  <si>
+    <t>1 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-24/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-24/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-24/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 10:13:23 AM</t>
+  </si>
+  <si>
+    <t>DN-18</t>
+  </si>
+  <si>
+    <t> | 25 min | 10:05 AM—10:30 AM |   DN-18</t>
+  </si>
+  <si>
+    <t> | 7 min | 10:09 AM—10:16 AM | Yellow Line | 10:09 AM from Dum Dum Cantonment | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>3.57x</t>
+  </si>
+  <si>
+    <t>72.0% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-25/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-25/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/10_00_AM/MC-25/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -990,6 +1579,48 @@
   </si>
   <si>
     <t>12:00 AM Savings (%)</t>
+  </si>
+  <si>
+    <t>10:00 AM Scraped At</t>
+  </si>
+  <si>
+    <t>10:00 AM Actual Bus</t>
+  </si>
+  <si>
+    <t>10:00 AM Bus Walk</t>
+  </si>
+  <si>
+    <t>10:00 AM Bus (min)</t>
+  </si>
+  <si>
+    <t>10:00 AM Bus Route</t>
+  </si>
+  <si>
+    <t>10:00 AM Bus Raw Details</t>
+  </si>
+  <si>
+    <t>10:00 AM Actual Metro</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Walk</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro (min)</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Route</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>10:00 AM Car (min)</t>
+  </si>
+  <si>
+    <t>10:00 AM Faster Mode</t>
+  </si>
+  <si>
+    <t>10:00 AM Savings (%)</t>
   </si>
 </sst>
 </file>
@@ -4043,10 +4674,2647 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R26"/>
+  <dimension ref="A1:AF26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:18" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s">
+        <v>313</v>
+      </c>
+      <c r="K2" t="s">
+        <v>314</v>
+      </c>
+      <c r="L2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M2" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2">
+        <v>50</v>
+      </c>
+      <c r="O2" t="s">
+        <v>45</v>
+      </c>
+      <c r="P2" t="s">
+        <v>315</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>47</v>
+      </c>
+      <c r="R2" t="s">
+        <v>44</v>
+      </c>
+      <c r="S2">
+        <v>28</v>
+      </c>
+      <c r="T2" t="s">
+        <v>48</v>
+      </c>
+      <c r="U2" t="s">
+        <v>316</v>
+      </c>
+      <c r="V2">
+        <v>51</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="X2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>317</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>318</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>320</v>
+      </c>
+      <c r="D3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J3" t="s">
+        <v>313</v>
+      </c>
+      <c r="K3" t="s">
+        <v>314</v>
+      </c>
+      <c r="L3" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" t="s">
+        <v>44</v>
+      </c>
+      <c r="N3">
+        <v>51</v>
+      </c>
+      <c r="O3" t="s">
+        <v>43</v>
+      </c>
+      <c r="P3" t="s">
+        <v>321</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>47</v>
+      </c>
+      <c r="R3" t="s">
+        <v>44</v>
+      </c>
+      <c r="S3">
+        <v>28</v>
+      </c>
+      <c r="T3" t="s">
+        <v>48</v>
+      </c>
+      <c r="U3" t="s">
+        <v>322</v>
+      </c>
+      <c r="V3">
+        <v>54</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="X3" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>323</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>324</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
+        <v>326</v>
+      </c>
+      <c r="D4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J4" t="s">
+        <v>313</v>
+      </c>
+      <c r="K4" t="s">
+        <v>314</v>
+      </c>
+      <c r="L4" t="s">
+        <v>327</v>
+      </c>
+      <c r="M4" t="s">
+        <v>44</v>
+      </c>
+      <c r="N4">
+        <v>12</v>
+      </c>
+      <c r="O4" t="s">
+        <v>43</v>
+      </c>
+      <c r="P4" t="s">
+        <v>328</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>47</v>
+      </c>
+      <c r="R4" t="s">
+        <v>44</v>
+      </c>
+      <c r="S4">
+        <v>7</v>
+      </c>
+      <c r="T4" t="s">
+        <v>48</v>
+      </c>
+      <c r="U4" t="s">
+        <v>329</v>
+      </c>
+      <c r="V4">
+        <v>15</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="X4" t="s">
+        <v>330</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>331</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>332</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>333</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>335</v>
+      </c>
+      <c r="D5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H5" t="s">
+        <v>74</v>
+      </c>
+      <c r="I5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" t="s">
+        <v>313</v>
+      </c>
+      <c r="K5" t="s">
+        <v>314</v>
+      </c>
+      <c r="L5" t="s">
+        <v>336</v>
+      </c>
+      <c r="M5" t="s">
+        <v>44</v>
+      </c>
+      <c r="N5">
+        <v>18</v>
+      </c>
+      <c r="O5" t="s">
+        <v>43</v>
+      </c>
+      <c r="P5" t="s">
+        <v>337</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>47</v>
+      </c>
+      <c r="R5" t="s">
+        <v>44</v>
+      </c>
+      <c r="S5">
+        <v>11</v>
+      </c>
+      <c r="T5" t="s">
+        <v>48</v>
+      </c>
+      <c r="U5" t="s">
+        <v>338</v>
+      </c>
+      <c r="V5">
+        <v>23</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="X5" t="s">
+        <v>91</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>92</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>339</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>340</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
+        <v>342</v>
+      </c>
+      <c r="D6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H6" t="s">
+        <v>98</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" t="s">
+        <v>313</v>
+      </c>
+      <c r="K6" t="s">
+        <v>314</v>
+      </c>
+      <c r="L6" t="s">
+        <v>99</v>
+      </c>
+      <c r="M6" t="s">
+        <v>44</v>
+      </c>
+      <c r="N6">
+        <v>18</v>
+      </c>
+      <c r="O6" t="s">
+        <v>43</v>
+      </c>
+      <c r="P6" t="s">
+        <v>343</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>47</v>
+      </c>
+      <c r="R6" t="s">
+        <v>44</v>
+      </c>
+      <c r="S6">
+        <v>11</v>
+      </c>
+      <c r="T6" t="s">
+        <v>48</v>
+      </c>
+      <c r="U6" t="s">
+        <v>344</v>
+      </c>
+      <c r="V6">
+        <v>18</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="X6" t="s">
+        <v>91</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>92</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>345</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>346</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>348</v>
+      </c>
+      <c r="D7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
+        <v>73</v>
+      </c>
+      <c r="J7" t="s">
+        <v>313</v>
+      </c>
+      <c r="K7" t="s">
+        <v>314</v>
+      </c>
+      <c r="L7" t="s">
+        <v>43</v>
+      </c>
+      <c r="M7" t="s">
+        <v>44</v>
+      </c>
+      <c r="N7">
+        <v>24</v>
+      </c>
+      <c r="O7" t="s">
+        <v>43</v>
+      </c>
+      <c r="P7" t="s">
+        <v>349</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>47</v>
+      </c>
+      <c r="R7" t="s">
+        <v>44</v>
+      </c>
+      <c r="S7">
+        <v>12</v>
+      </c>
+      <c r="T7" t="s">
+        <v>48</v>
+      </c>
+      <c r="U7" t="s">
+        <v>350</v>
+      </c>
+      <c r="V7">
+        <v>32</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="X7" t="s">
+        <v>110</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>351</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>352</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
+        <v>354</v>
+      </c>
+      <c r="D8" t="s">
+        <v>116</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>72</v>
+      </c>
+      <c r="H8" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" t="s">
+        <v>117</v>
+      </c>
+      <c r="J8" t="s">
+        <v>313</v>
+      </c>
+      <c r="K8" t="s">
+        <v>314</v>
+      </c>
+      <c r="L8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M8" t="s">
+        <v>44</v>
+      </c>
+      <c r="N8">
+        <v>27</v>
+      </c>
+      <c r="O8" t="s">
+        <v>43</v>
+      </c>
+      <c r="P8" t="s">
+        <v>355</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>47</v>
+      </c>
+      <c r="R8" t="s">
+        <v>44</v>
+      </c>
+      <c r="S8">
+        <v>17</v>
+      </c>
+      <c r="T8" t="s">
+        <v>48</v>
+      </c>
+      <c r="U8" t="s">
+        <v>356</v>
+      </c>
+      <c r="V8">
+        <v>29</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="X8" t="s">
+        <v>357</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>358</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>359</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>360</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
+        <v>362</v>
+      </c>
+      <c r="D9" t="s">
+        <v>129</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" t="s">
+        <v>72</v>
+      </c>
+      <c r="H9" t="s">
+        <v>117</v>
+      </c>
+      <c r="I9" t="s">
+        <v>130</v>
+      </c>
+      <c r="J9" t="s">
+        <v>313</v>
+      </c>
+      <c r="K9" t="s">
+        <v>314</v>
+      </c>
+      <c r="L9" t="s">
+        <v>61</v>
+      </c>
+      <c r="M9" t="s">
+        <v>44</v>
+      </c>
+      <c r="N9">
+        <v>22</v>
+      </c>
+      <c r="O9" t="s">
+        <v>43</v>
+      </c>
+      <c r="P9" t="s">
+        <v>363</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>47</v>
+      </c>
+      <c r="R9" t="s">
+        <v>44</v>
+      </c>
+      <c r="S9">
+        <v>15</v>
+      </c>
+      <c r="T9" t="s">
+        <v>48</v>
+      </c>
+      <c r="U9" t="s">
+        <v>364</v>
+      </c>
+      <c r="V9">
+        <v>25</v>
+      </c>
+      <c r="W9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="X9" t="s">
+        <v>133</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>134</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>365</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>366</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>368</v>
+      </c>
+      <c r="D10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" t="s">
+        <v>72</v>
+      </c>
+      <c r="H10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I10" t="s">
+        <v>40</v>
+      </c>
+      <c r="J10" t="s">
+        <v>313</v>
+      </c>
+      <c r="K10" t="s">
+        <v>314</v>
+      </c>
+      <c r="L10" t="s">
+        <v>140</v>
+      </c>
+      <c r="M10" t="s">
+        <v>44</v>
+      </c>
+      <c r="N10">
+        <v>36</v>
+      </c>
+      <c r="O10" t="s">
+        <v>141</v>
+      </c>
+      <c r="P10" t="s">
+        <v>369</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>47</v>
+      </c>
+      <c r="R10" t="s">
+        <v>44</v>
+      </c>
+      <c r="S10">
+        <v>16</v>
+      </c>
+      <c r="T10" t="s">
+        <v>48</v>
+      </c>
+      <c r="U10" t="s">
+        <v>370</v>
+      </c>
+      <c r="V10">
+        <v>38</v>
+      </c>
+      <c r="W10" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="X10" t="s">
+        <v>145</v>
+      </c>
+      <c r="Y10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>146</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>371</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>372</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" t="s">
+        <v>374</v>
+      </c>
+      <c r="D11" t="s">
+        <v>151</v>
+      </c>
+      <c r="E11" t="s">
+        <v>152</v>
+      </c>
+      <c r="F11" t="s">
+        <v>153</v>
+      </c>
+      <c r="G11" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" t="s">
+        <v>154</v>
+      </c>
+      <c r="I11" t="s">
+        <v>155</v>
+      </c>
+      <c r="J11" t="s">
+        <v>313</v>
+      </c>
+      <c r="K11" t="s">
+        <v>314</v>
+      </c>
+      <c r="L11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M11" t="s">
+        <v>44</v>
+      </c>
+      <c r="N11">
+        <v>40</v>
+      </c>
+      <c r="O11" t="s">
+        <v>43</v>
+      </c>
+      <c r="P11" t="s">
+        <v>375</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>157</v>
+      </c>
+      <c r="R11" t="s">
+        <v>44</v>
+      </c>
+      <c r="S11">
+        <v>30</v>
+      </c>
+      <c r="T11" t="s">
+        <v>48</v>
+      </c>
+      <c r="U11" t="s">
+        <v>376</v>
+      </c>
+      <c r="V11">
+        <v>52</v>
+      </c>
+      <c r="W11" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="X11" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>377</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>378</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>379</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s">
+        <v>381</v>
+      </c>
+      <c r="D12" t="s">
+        <v>167</v>
+      </c>
+      <c r="E12" t="s">
+        <v>152</v>
+      </c>
+      <c r="F12" t="s">
+        <v>153</v>
+      </c>
+      <c r="G12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H12" t="s">
+        <v>168</v>
+      </c>
+      <c r="I12" t="s">
+        <v>155</v>
+      </c>
+      <c r="J12" t="s">
+        <v>313</v>
+      </c>
+      <c r="K12" t="s">
+        <v>314</v>
+      </c>
+      <c r="L12" t="s">
+        <v>382</v>
+      </c>
+      <c r="M12" t="s">
+        <v>44</v>
+      </c>
+      <c r="N12">
+        <v>26</v>
+      </c>
+      <c r="O12" t="s">
+        <v>43</v>
+      </c>
+      <c r="P12" t="s">
+        <v>383</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>157</v>
+      </c>
+      <c r="R12" t="s">
+        <v>44</v>
+      </c>
+      <c r="S12">
+        <v>21</v>
+      </c>
+      <c r="T12" t="s">
+        <v>48</v>
+      </c>
+      <c r="U12" t="s">
+        <v>384</v>
+      </c>
+      <c r="V12">
+        <v>33</v>
+      </c>
+      <c r="W12" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="X12" t="s">
+        <v>385</v>
+      </c>
+      <c r="Y12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>386</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>387</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>388</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" t="s">
+        <v>390</v>
+      </c>
+      <c r="D13" t="s">
+        <v>178</v>
+      </c>
+      <c r="E13" t="s">
+        <v>152</v>
+      </c>
+      <c r="F13" t="s">
+        <v>179</v>
+      </c>
+      <c r="G13" t="s">
+        <v>72</v>
+      </c>
+      <c r="H13" t="s">
+        <v>154</v>
+      </c>
+      <c r="I13" t="s">
+        <v>168</v>
+      </c>
+      <c r="J13" t="s">
+        <v>313</v>
+      </c>
+      <c r="K13" t="s">
+        <v>314</v>
+      </c>
+      <c r="L13" t="s">
+        <v>391</v>
+      </c>
+      <c r="M13" t="s">
+        <v>44</v>
+      </c>
+      <c r="N13">
+        <v>27</v>
+      </c>
+      <c r="O13" t="s">
+        <v>392</v>
+      </c>
+      <c r="P13" t="s">
+        <v>393</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>157</v>
+      </c>
+      <c r="R13" t="s">
+        <v>44</v>
+      </c>
+      <c r="S13">
+        <v>11</v>
+      </c>
+      <c r="T13" t="s">
+        <v>48</v>
+      </c>
+      <c r="U13" t="s">
+        <v>394</v>
+      </c>
+      <c r="V13">
+        <v>30</v>
+      </c>
+      <c r="W13" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="X13" t="s">
+        <v>395</v>
+      </c>
+      <c r="Y13" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>396</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>397</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>398</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
+        <v>400</v>
+      </c>
+      <c r="D14" t="s">
+        <v>189</v>
+      </c>
+      <c r="E14" t="s">
+        <v>152</v>
+      </c>
+      <c r="F14" t="s">
+        <v>179</v>
+      </c>
+      <c r="G14" t="s">
+        <v>72</v>
+      </c>
+      <c r="H14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I14" t="s">
+        <v>155</v>
+      </c>
+      <c r="J14" t="s">
+        <v>313</v>
+      </c>
+      <c r="K14" t="s">
+        <v>314</v>
+      </c>
+      <c r="L14" t="s">
+        <v>191</v>
+      </c>
+      <c r="M14" t="s">
+        <v>44</v>
+      </c>
+      <c r="N14">
+        <v>26</v>
+      </c>
+      <c r="O14" t="s">
+        <v>45</v>
+      </c>
+      <c r="P14" t="s">
+        <v>401</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>157</v>
+      </c>
+      <c r="R14" t="s">
+        <v>44</v>
+      </c>
+      <c r="S14">
+        <v>18</v>
+      </c>
+      <c r="T14" t="s">
+        <v>48</v>
+      </c>
+      <c r="U14" t="s">
+        <v>402</v>
+      </c>
+      <c r="V14">
+        <v>24</v>
+      </c>
+      <c r="W14" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="X14" t="s">
+        <v>404</v>
+      </c>
+      <c r="Y14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>405</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>406</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>407</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>409</v>
+      </c>
+      <c r="D15" t="s">
+        <v>201</v>
+      </c>
+      <c r="E15" t="s">
+        <v>152</v>
+      </c>
+      <c r="F15" t="s">
+        <v>153</v>
+      </c>
+      <c r="G15" t="s">
+        <v>72</v>
+      </c>
+      <c r="H15" t="s">
+        <v>154</v>
+      </c>
+      <c r="I15" t="s">
+        <v>190</v>
+      </c>
+      <c r="J15" t="s">
+        <v>313</v>
+      </c>
+      <c r="K15" t="s">
+        <v>314</v>
+      </c>
+      <c r="L15" t="s">
+        <v>43</v>
+      </c>
+      <c r="M15" t="s">
+        <v>44</v>
+      </c>
+      <c r="N15">
+        <v>29</v>
+      </c>
+      <c r="O15" t="s">
+        <v>43</v>
+      </c>
+      <c r="P15" t="s">
+        <v>410</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>157</v>
+      </c>
+      <c r="R15" t="s">
+        <v>44</v>
+      </c>
+      <c r="S15">
+        <v>12</v>
+      </c>
+      <c r="T15" t="s">
+        <v>48</v>
+      </c>
+      <c r="U15" t="s">
+        <v>411</v>
+      </c>
+      <c r="V15">
+        <v>30</v>
+      </c>
+      <c r="W15" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="X15" t="s">
+        <v>413</v>
+      </c>
+      <c r="Y15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>414</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>415</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>416</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s">
+        <v>418</v>
+      </c>
+      <c r="D16" t="s">
+        <v>211</v>
+      </c>
+      <c r="E16" t="s">
+        <v>152</v>
+      </c>
+      <c r="F16" t="s">
+        <v>153</v>
+      </c>
+      <c r="G16" t="s">
+        <v>72</v>
+      </c>
+      <c r="H16" t="s">
+        <v>40</v>
+      </c>
+      <c r="I16" t="s">
+        <v>155</v>
+      </c>
+      <c r="J16" t="s">
+        <v>313</v>
+      </c>
+      <c r="K16" t="s">
+        <v>314</v>
+      </c>
+      <c r="L16" t="s">
+        <v>43</v>
+      </c>
+      <c r="M16" t="s">
+        <v>44</v>
+      </c>
+      <c r="N16">
+        <v>34</v>
+      </c>
+      <c r="O16" t="s">
+        <v>43</v>
+      </c>
+      <c r="P16" t="s">
+        <v>419</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>157</v>
+      </c>
+      <c r="R16" t="s">
+        <v>44</v>
+      </c>
+      <c r="S16">
+        <v>25</v>
+      </c>
+      <c r="T16" t="s">
+        <v>48</v>
+      </c>
+      <c r="U16" t="s">
+        <v>420</v>
+      </c>
+      <c r="V16">
+        <v>39</v>
+      </c>
+      <c r="W16" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="X16" t="s">
+        <v>215</v>
+      </c>
+      <c r="Y16" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>421</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>422</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>423</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" t="s">
+        <v>425</v>
+      </c>
+      <c r="D17" t="s">
+        <v>221</v>
+      </c>
+      <c r="E17" t="s">
+        <v>222</v>
+      </c>
+      <c r="F17" t="s">
+        <v>223</v>
+      </c>
+      <c r="G17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H17" t="s">
+        <v>130</v>
+      </c>
+      <c r="I17" t="s">
+        <v>224</v>
+      </c>
+      <c r="J17" t="s">
+        <v>313</v>
+      </c>
+      <c r="K17" t="s">
+        <v>314</v>
+      </c>
+      <c r="L17" t="s">
+        <v>426</v>
+      </c>
+      <c r="M17" t="s">
+        <v>44</v>
+      </c>
+      <c r="N17">
+        <v>36</v>
+      </c>
+      <c r="O17" t="s">
+        <v>43</v>
+      </c>
+      <c r="P17" t="s">
+        <v>427</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>428</v>
+      </c>
+      <c r="R17" t="s">
+        <v>44</v>
+      </c>
+      <c r="S17">
+        <v>23</v>
+      </c>
+      <c r="T17" t="s">
+        <v>48</v>
+      </c>
+      <c r="U17" t="s">
+        <v>429</v>
+      </c>
+      <c r="V17">
+        <v>36</v>
+      </c>
+      <c r="W17" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="X17" t="s">
+        <v>431</v>
+      </c>
+      <c r="Y17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>432</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>433</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>434</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="s">
+        <v>436</v>
+      </c>
+      <c r="D18" t="s">
+        <v>231</v>
+      </c>
+      <c r="E18" t="s">
+        <v>222</v>
+      </c>
+      <c r="F18" t="s">
+        <v>179</v>
+      </c>
+      <c r="G18" t="s">
+        <v>72</v>
+      </c>
+      <c r="H18" t="s">
+        <v>232</v>
+      </c>
+      <c r="I18" t="s">
+        <v>224</v>
+      </c>
+      <c r="J18" t="s">
+        <v>313</v>
+      </c>
+      <c r="K18" t="s">
+        <v>314</v>
+      </c>
+      <c r="L18" t="s">
+        <v>233</v>
+      </c>
+      <c r="M18" t="s">
+        <v>44</v>
+      </c>
+      <c r="N18">
+        <v>16</v>
+      </c>
+      <c r="O18" t="s">
+        <v>43</v>
+      </c>
+      <c r="P18" t="s">
+        <v>437</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>428</v>
+      </c>
+      <c r="R18" t="s">
+        <v>44</v>
+      </c>
+      <c r="S18">
+        <v>12</v>
+      </c>
+      <c r="T18" t="s">
+        <v>48</v>
+      </c>
+      <c r="U18" t="s">
+        <v>438</v>
+      </c>
+      <c r="V18">
+        <v>22</v>
+      </c>
+      <c r="W18" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="X18" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>377</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>440</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>441</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" t="s">
+        <v>443</v>
+      </c>
+      <c r="D19" t="s">
+        <v>238</v>
+      </c>
+      <c r="E19" t="s">
+        <v>222</v>
+      </c>
+      <c r="F19" t="s">
+        <v>223</v>
+      </c>
+      <c r="G19" t="s">
+        <v>72</v>
+      </c>
+      <c r="H19" t="s">
+        <v>130</v>
+      </c>
+      <c r="I19" t="s">
+        <v>239</v>
+      </c>
+      <c r="J19" t="s">
+        <v>313</v>
+      </c>
+      <c r="K19" t="s">
+        <v>314</v>
+      </c>
+      <c r="L19" t="s">
+        <v>444</v>
+      </c>
+      <c r="M19" t="s">
+        <v>44</v>
+      </c>
+      <c r="N19">
+        <v>47</v>
+      </c>
+      <c r="O19" t="s">
+        <v>119</v>
+      </c>
+      <c r="P19" t="s">
+        <v>445</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>428</v>
+      </c>
+      <c r="R19" t="s">
+        <v>44</v>
+      </c>
+      <c r="S19">
+        <v>19</v>
+      </c>
+      <c r="T19" t="s">
+        <v>48</v>
+      </c>
+      <c r="U19" t="s">
+        <v>446</v>
+      </c>
+      <c r="V19">
+        <v>30</v>
+      </c>
+      <c r="W19" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="X19" t="s">
+        <v>448</v>
+      </c>
+      <c r="Y19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>449</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>450</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>451</v>
+      </c>
+      <c r="AF19" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" t="s">
+        <v>453</v>
+      </c>
+      <c r="D20" t="s">
+        <v>245</v>
+      </c>
+      <c r="E20" t="s">
+        <v>246</v>
+      </c>
+      <c r="F20" t="s">
+        <v>247</v>
+      </c>
+      <c r="G20" t="s">
+        <v>38</v>
+      </c>
+      <c r="H20" t="s">
+        <v>248</v>
+      </c>
+      <c r="I20" t="s">
+        <v>249</v>
+      </c>
+      <c r="J20" t="s">
+        <v>313</v>
+      </c>
+      <c r="K20" t="s">
+        <v>314</v>
+      </c>
+      <c r="L20" t="s">
+        <v>250</v>
+      </c>
+      <c r="M20" t="s">
+        <v>44</v>
+      </c>
+      <c r="N20">
+        <v>26</v>
+      </c>
+      <c r="O20" t="s">
+        <v>43</v>
+      </c>
+      <c r="P20" t="s">
+        <v>454</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>455</v>
+      </c>
+      <c r="R20" t="s">
+        <v>44</v>
+      </c>
+      <c r="S20">
+        <v>17</v>
+      </c>
+      <c r="T20" t="s">
+        <v>48</v>
+      </c>
+      <c r="U20" t="s">
+        <v>456</v>
+      </c>
+      <c r="V20">
+        <v>27</v>
+      </c>
+      <c r="W20" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="X20" t="s">
+        <v>457</v>
+      </c>
+      <c r="Y20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>459</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>460</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" t="s">
+        <v>462</v>
+      </c>
+      <c r="D21" t="s">
+        <v>255</v>
+      </c>
+      <c r="E21" t="s">
+        <v>246</v>
+      </c>
+      <c r="F21" t="s">
+        <v>179</v>
+      </c>
+      <c r="G21" t="s">
+        <v>72</v>
+      </c>
+      <c r="H21" t="s">
+        <v>256</v>
+      </c>
+      <c r="I21" t="s">
+        <v>249</v>
+      </c>
+      <c r="J21" t="s">
+        <v>313</v>
+      </c>
+      <c r="K21" t="s">
+        <v>314</v>
+      </c>
+      <c r="L21" t="s">
+        <v>463</v>
+      </c>
+      <c r="M21" t="s">
+        <v>44</v>
+      </c>
+      <c r="N21">
+        <v>12</v>
+      </c>
+      <c r="O21" t="s">
+        <v>43</v>
+      </c>
+      <c r="P21" t="s">
+        <v>464</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>455</v>
+      </c>
+      <c r="R21" t="s">
+        <v>44</v>
+      </c>
+      <c r="S21">
+        <v>9</v>
+      </c>
+      <c r="T21" t="s">
+        <v>48</v>
+      </c>
+      <c r="U21" t="s">
+        <v>465</v>
+      </c>
+      <c r="V21">
+        <v>15</v>
+      </c>
+      <c r="W21" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="X21" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y21" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>377</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>466</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>467</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" t="s">
+        <v>469</v>
+      </c>
+      <c r="D22" t="s">
+        <v>261</v>
+      </c>
+      <c r="E22" t="s">
+        <v>246</v>
+      </c>
+      <c r="F22" t="s">
+        <v>179</v>
+      </c>
+      <c r="G22" t="s">
+        <v>72</v>
+      </c>
+      <c r="H22" t="s">
+        <v>248</v>
+      </c>
+      <c r="I22" t="s">
+        <v>256</v>
+      </c>
+      <c r="J22" t="s">
+        <v>313</v>
+      </c>
+      <c r="K22" t="s">
+        <v>314</v>
+      </c>
+      <c r="L22" t="s">
+        <v>250</v>
+      </c>
+      <c r="M22" t="s">
+        <v>44</v>
+      </c>
+      <c r="N22">
+        <v>14</v>
+      </c>
+      <c r="O22" t="s">
+        <v>43</v>
+      </c>
+      <c r="P22" t="s">
+        <v>470</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>455</v>
+      </c>
+      <c r="R22" t="s">
+        <v>44</v>
+      </c>
+      <c r="S22">
+        <v>8</v>
+      </c>
+      <c r="T22" t="s">
+        <v>48</v>
+      </c>
+      <c r="U22" t="s">
+        <v>471</v>
+      </c>
+      <c r="V22">
+        <v>12</v>
+      </c>
+      <c r="W22" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="X22" t="s">
+        <v>473</v>
+      </c>
+      <c r="Y22" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>474</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>475</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>476</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" t="s">
+        <v>478</v>
+      </c>
+      <c r="D23" t="s">
+        <v>271</v>
+      </c>
+      <c r="E23" t="s">
+        <v>246</v>
+      </c>
+      <c r="F23" t="s">
+        <v>247</v>
+      </c>
+      <c r="G23" t="s">
+        <v>72</v>
+      </c>
+      <c r="H23" t="s">
+        <v>248</v>
+      </c>
+      <c r="I23" t="s">
+        <v>272</v>
+      </c>
+      <c r="J23" t="s">
+        <v>313</v>
+      </c>
+      <c r="K23" t="s">
+        <v>314</v>
+      </c>
+      <c r="L23" t="s">
+        <v>250</v>
+      </c>
+      <c r="M23" t="s">
+        <v>44</v>
+      </c>
+      <c r="N23">
+        <v>22</v>
+      </c>
+      <c r="O23" t="s">
+        <v>43</v>
+      </c>
+      <c r="P23" t="s">
+        <v>479</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>455</v>
+      </c>
+      <c r="R23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S23">
+        <v>14</v>
+      </c>
+      <c r="T23" t="s">
+        <v>48</v>
+      </c>
+      <c r="U23" t="s">
+        <v>480</v>
+      </c>
+      <c r="V23">
+        <v>21</v>
+      </c>
+      <c r="W23" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="X23" t="s">
+        <v>431</v>
+      </c>
+      <c r="Y23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>481</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>482</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>483</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" t="s">
+        <v>485</v>
+      </c>
+      <c r="D24" t="s">
+        <v>277</v>
+      </c>
+      <c r="E24" t="s">
+        <v>246</v>
+      </c>
+      <c r="F24" t="s">
+        <v>247</v>
+      </c>
+      <c r="G24" t="s">
+        <v>72</v>
+      </c>
+      <c r="H24" t="s">
+        <v>256</v>
+      </c>
+      <c r="I24" t="s">
+        <v>272</v>
+      </c>
+      <c r="J24" t="s">
+        <v>313</v>
+      </c>
+      <c r="K24" t="s">
+        <v>314</v>
+      </c>
+      <c r="L24" t="s">
+        <v>463</v>
+      </c>
+      <c r="M24" t="s">
+        <v>44</v>
+      </c>
+      <c r="N24">
+        <v>8</v>
+      </c>
+      <c r="O24" t="s">
+        <v>43</v>
+      </c>
+      <c r="P24" t="s">
+        <v>486</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>455</v>
+      </c>
+      <c r="R24" t="s">
+        <v>44</v>
+      </c>
+      <c r="S24">
+        <v>6</v>
+      </c>
+      <c r="T24" t="s">
+        <v>48</v>
+      </c>
+      <c r="U24" t="s">
+        <v>487</v>
+      </c>
+      <c r="V24">
+        <v>9</v>
+      </c>
+      <c r="W24" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="X24" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y24" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>377</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>489</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>490</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" t="s">
+        <v>492</v>
+      </c>
+      <c r="D25" t="s">
+        <v>287</v>
+      </c>
+      <c r="E25" t="s">
+        <v>246</v>
+      </c>
+      <c r="F25" t="s">
+        <v>247</v>
+      </c>
+      <c r="G25" t="s">
+        <v>72</v>
+      </c>
+      <c r="H25" t="s">
+        <v>272</v>
+      </c>
+      <c r="I25" t="s">
+        <v>249</v>
+      </c>
+      <c r="J25" t="s">
+        <v>313</v>
+      </c>
+      <c r="K25" t="s">
+        <v>314</v>
+      </c>
+      <c r="L25" t="s">
+        <v>43</v>
+      </c>
+      <c r="M25" t="s">
+        <v>44</v>
+      </c>
+      <c r="N25">
+        <v>4</v>
+      </c>
+      <c r="O25" t="s">
+        <v>43</v>
+      </c>
+      <c r="P25" t="s">
+        <v>493</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>455</v>
+      </c>
+      <c r="R25" t="s">
+        <v>44</v>
+      </c>
+      <c r="S25">
+        <v>3</v>
+      </c>
+      <c r="T25" t="s">
+        <v>48</v>
+      </c>
+      <c r="U25" t="s">
+        <v>494</v>
+      </c>
+      <c r="V25">
+        <v>6</v>
+      </c>
+      <c r="W25" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="X25" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y25" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>377</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>496</v>
+      </c>
+      <c r="AE25" t="s">
+        <v>497</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" t="s">
+        <v>499</v>
+      </c>
+      <c r="D26" t="s">
+        <v>297</v>
+      </c>
+      <c r="E26" t="s">
+        <v>298</v>
+      </c>
+      <c r="F26" t="s">
+        <v>299</v>
+      </c>
+      <c r="G26" t="s">
+        <v>72</v>
+      </c>
+      <c r="H26" t="s">
+        <v>300</v>
+      </c>
+      <c r="I26" t="s">
+        <v>301</v>
+      </c>
+      <c r="J26" t="s">
+        <v>313</v>
+      </c>
+      <c r="K26" t="s">
+        <v>314</v>
+      </c>
+      <c r="L26" t="s">
+        <v>500</v>
+      </c>
+      <c r="M26" t="s">
+        <v>44</v>
+      </c>
+      <c r="N26">
+        <v>25</v>
+      </c>
+      <c r="O26" t="s">
+        <v>119</v>
+      </c>
+      <c r="P26" t="s">
+        <v>501</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>304</v>
+      </c>
+      <c r="R26" t="s">
+        <v>44</v>
+      </c>
+      <c r="S26">
+        <v>7</v>
+      </c>
+      <c r="T26" t="s">
+        <v>48</v>
+      </c>
+      <c r="U26" t="s">
+        <v>502</v>
+      </c>
+      <c r="V26">
+        <v>16</v>
+      </c>
+      <c r="W26" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="X26" t="s">
+        <v>503</v>
+      </c>
+      <c r="Y26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>504</v>
+      </c>
+      <c r="AA26" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC26" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD26" t="s">
+        <v>505</v>
+      </c>
+      <c r="AE26" t="s">
+        <v>506</v>
+      </c>
+      <c r="AF26" t="s">
+        <v>507</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AF1"/>
+  <hyperlinks>
+    <hyperlink ref="AA2" r:id="rId1"/>
+    <hyperlink ref="AB2" r:id="rId2"/>
+    <hyperlink ref="AC2" r:id="rId3"/>
+    <hyperlink ref="AA3" r:id="rId4"/>
+    <hyperlink ref="AB3" r:id="rId5"/>
+    <hyperlink ref="AC3" r:id="rId6"/>
+    <hyperlink ref="AA4" r:id="rId7"/>
+    <hyperlink ref="AB4" r:id="rId8"/>
+    <hyperlink ref="AC4" r:id="rId9"/>
+    <hyperlink ref="AA5" r:id="rId10"/>
+    <hyperlink ref="AB5" r:id="rId11"/>
+    <hyperlink ref="AC5" r:id="rId12"/>
+    <hyperlink ref="AA6" r:id="rId13"/>
+    <hyperlink ref="AB6" r:id="rId14"/>
+    <hyperlink ref="AC6" r:id="rId15"/>
+    <hyperlink ref="AA7" r:id="rId16"/>
+    <hyperlink ref="AB7" r:id="rId17"/>
+    <hyperlink ref="AC7" r:id="rId18"/>
+    <hyperlink ref="AA8" r:id="rId19"/>
+    <hyperlink ref="AB8" r:id="rId20"/>
+    <hyperlink ref="AC8" r:id="rId21"/>
+    <hyperlink ref="AA9" r:id="rId22"/>
+    <hyperlink ref="AB9" r:id="rId23"/>
+    <hyperlink ref="AC9" r:id="rId24"/>
+    <hyperlink ref="AA10" r:id="rId25"/>
+    <hyperlink ref="AB10" r:id="rId26"/>
+    <hyperlink ref="AC10" r:id="rId27"/>
+    <hyperlink ref="AA11" r:id="rId28"/>
+    <hyperlink ref="AB11" r:id="rId29"/>
+    <hyperlink ref="AC11" r:id="rId30"/>
+    <hyperlink ref="AA12" r:id="rId31"/>
+    <hyperlink ref="AB12" r:id="rId32"/>
+    <hyperlink ref="AC12" r:id="rId33"/>
+    <hyperlink ref="AA13" r:id="rId34"/>
+    <hyperlink ref="AB13" r:id="rId35"/>
+    <hyperlink ref="AC13" r:id="rId36"/>
+    <hyperlink ref="AA14" r:id="rId37"/>
+    <hyperlink ref="AB14" r:id="rId38"/>
+    <hyperlink ref="AC14" r:id="rId39"/>
+    <hyperlink ref="AA15" r:id="rId40"/>
+    <hyperlink ref="AB15" r:id="rId41"/>
+    <hyperlink ref="AC15" r:id="rId42"/>
+    <hyperlink ref="AA16" r:id="rId43"/>
+    <hyperlink ref="AB16" r:id="rId44"/>
+    <hyperlink ref="AC16" r:id="rId45"/>
+    <hyperlink ref="AA17" r:id="rId46"/>
+    <hyperlink ref="AB17" r:id="rId47"/>
+    <hyperlink ref="AC17" r:id="rId48"/>
+    <hyperlink ref="AA18" r:id="rId49"/>
+    <hyperlink ref="AB18" r:id="rId50"/>
+    <hyperlink ref="AC18" r:id="rId51"/>
+    <hyperlink ref="AA19" r:id="rId52"/>
+    <hyperlink ref="AB19" r:id="rId53"/>
+    <hyperlink ref="AC19" r:id="rId54"/>
+    <hyperlink ref="AA20" r:id="rId55"/>
+    <hyperlink ref="AB20" r:id="rId56"/>
+    <hyperlink ref="AC20" r:id="rId57"/>
+    <hyperlink ref="AA21" r:id="rId58"/>
+    <hyperlink ref="AB21" r:id="rId59"/>
+    <hyperlink ref="AC21" r:id="rId60"/>
+    <hyperlink ref="AA22" r:id="rId61"/>
+    <hyperlink ref="AB22" r:id="rId62"/>
+    <hyperlink ref="AC22" r:id="rId63"/>
+    <hyperlink ref="AA23" r:id="rId64"/>
+    <hyperlink ref="AB23" r:id="rId65"/>
+    <hyperlink ref="AC23" r:id="rId66"/>
+    <hyperlink ref="AA24" r:id="rId67"/>
+    <hyperlink ref="AB24" r:id="rId68"/>
+    <hyperlink ref="AC24" r:id="rId69"/>
+    <hyperlink ref="AA25" r:id="rId70"/>
+    <hyperlink ref="AB25" r:id="rId71"/>
+    <hyperlink ref="AC25" r:id="rId72"/>
+    <hyperlink ref="AA26" r:id="rId73"/>
+    <hyperlink ref="AB26" r:id="rId74"/>
+    <hyperlink ref="AC26" r:id="rId75"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AF26"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:32" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>3</v>
       </c>
@@ -4060,49 +7328,91 @@
         <v>8</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>312</v>
+        <v>508</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>313</v>
+        <v>509</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>314</v>
+        <v>510</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>315</v>
+        <v>511</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>316</v>
+        <v>512</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>317</v>
+        <v>513</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>318</v>
+        <v>514</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>319</v>
+        <v>515</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>320</v>
+        <v>516</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>321</v>
+        <v>517</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>322</v>
+        <v>518</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>323</v>
+        <v>519</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>324</v>
+        <v>520</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>325</v>
+        <v>521</v>
+      </c>
+      <c r="S1" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>525</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>526</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="Y1" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="Z1" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="AA1" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="AB1" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="AC1" s="5" t="s">
+        <v>532</v>
+      </c>
+      <c r="AD1" s="5" t="s">
+        <v>533</v>
+      </c>
+      <c r="AE1" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="AF1" s="5" t="s">
+        <v>535</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>35</v>
       </c>
@@ -4157,8 +7467,50 @@
       <c r="R2" t="s">
         <v>52</v>
       </c>
+      <c r="S2" t="s">
+        <v>312</v>
+      </c>
+      <c r="T2" t="s">
+        <v>43</v>
+      </c>
+      <c r="U2" t="s">
+        <v>44</v>
+      </c>
+      <c r="V2">
+        <v>50</v>
+      </c>
+      <c r="W2" t="s">
+        <v>45</v>
+      </c>
+      <c r="X2" t="s">
+        <v>315</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA2">
+        <v>28</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>316</v>
+      </c>
+      <c r="AD2">
+        <v>51</v>
+      </c>
+      <c r="AE2" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -4213,8 +7565,50 @@
       <c r="R3" t="s">
         <v>66</v>
       </c>
+      <c r="S3" t="s">
+        <v>320</v>
+      </c>
+      <c r="T3" t="s">
+        <v>61</v>
+      </c>
+      <c r="U3" t="s">
+        <v>44</v>
+      </c>
+      <c r="V3">
+        <v>51</v>
+      </c>
+      <c r="W3" t="s">
+        <v>43</v>
+      </c>
+      <c r="X3" t="s">
+        <v>321</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA3">
+        <v>28</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>322</v>
+      </c>
+      <c r="AD3">
+        <v>54</v>
+      </c>
+      <c r="AE3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>66</v>
+      </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -4269,8 +7663,50 @@
       <c r="R4" t="s">
         <v>81</v>
       </c>
+      <c r="S4" t="s">
+        <v>326</v>
+      </c>
+      <c r="T4" t="s">
+        <v>327</v>
+      </c>
+      <c r="U4" t="s">
+        <v>44</v>
+      </c>
+      <c r="V4">
+        <v>12</v>
+      </c>
+      <c r="W4" t="s">
+        <v>43</v>
+      </c>
+      <c r="X4" t="s">
+        <v>328</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA4">
+        <v>7</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>329</v>
+      </c>
+      <c r="AD4">
+        <v>15</v>
+      </c>
+      <c r="AE4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>331</v>
+      </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>86</v>
       </c>
@@ -4325,8 +7761,50 @@
       <c r="R5" t="s">
         <v>92</v>
       </c>
+      <c r="S5" t="s">
+        <v>335</v>
+      </c>
+      <c r="T5" t="s">
+        <v>336</v>
+      </c>
+      <c r="U5" t="s">
+        <v>44</v>
+      </c>
+      <c r="V5">
+        <v>18</v>
+      </c>
+      <c r="W5" t="s">
+        <v>43</v>
+      </c>
+      <c r="X5" t="s">
+        <v>337</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA5">
+        <v>11</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>338</v>
+      </c>
+      <c r="AD5">
+        <v>23</v>
+      </c>
+      <c r="AE5" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>92</v>
+      </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>97</v>
       </c>
@@ -4381,8 +7859,50 @@
       <c r="R6" t="s">
         <v>92</v>
       </c>
+      <c r="S6" t="s">
+        <v>342</v>
+      </c>
+      <c r="T6" t="s">
+        <v>99</v>
+      </c>
+      <c r="U6" t="s">
+        <v>44</v>
+      </c>
+      <c r="V6">
+        <v>18</v>
+      </c>
+      <c r="W6" t="s">
+        <v>43</v>
+      </c>
+      <c r="X6" t="s">
+        <v>343</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA6">
+        <v>11</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>344</v>
+      </c>
+      <c r="AD6">
+        <v>18</v>
+      </c>
+      <c r="AE6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>92</v>
+      </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>106</v>
       </c>
@@ -4437,8 +7957,50 @@
       <c r="R7" t="s">
         <v>111</v>
       </c>
+      <c r="S7" t="s">
+        <v>348</v>
+      </c>
+      <c r="T7" t="s">
+        <v>43</v>
+      </c>
+      <c r="U7" t="s">
+        <v>44</v>
+      </c>
+      <c r="V7">
+        <v>24</v>
+      </c>
+      <c r="W7" t="s">
+        <v>43</v>
+      </c>
+      <c r="X7" t="s">
+        <v>349</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA7">
+        <v>12</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>350</v>
+      </c>
+      <c r="AD7">
+        <v>32</v>
+      </c>
+      <c r="AE7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>111</v>
+      </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>116</v>
       </c>
@@ -4493,8 +8055,50 @@
       <c r="R8" t="s">
         <v>124</v>
       </c>
+      <c r="S8" t="s">
+        <v>354</v>
+      </c>
+      <c r="T8" t="s">
+        <v>43</v>
+      </c>
+      <c r="U8" t="s">
+        <v>44</v>
+      </c>
+      <c r="V8">
+        <v>27</v>
+      </c>
+      <c r="W8" t="s">
+        <v>43</v>
+      </c>
+      <c r="X8" t="s">
+        <v>355</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA8">
+        <v>17</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>356</v>
+      </c>
+      <c r="AD8">
+        <v>29</v>
+      </c>
+      <c r="AE8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>358</v>
+      </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>129</v>
       </c>
@@ -4549,8 +8153,50 @@
       <c r="R9" t="s">
         <v>134</v>
       </c>
+      <c r="S9" t="s">
+        <v>362</v>
+      </c>
+      <c r="T9" t="s">
+        <v>61</v>
+      </c>
+      <c r="U9" t="s">
+        <v>44</v>
+      </c>
+      <c r="V9">
+        <v>22</v>
+      </c>
+      <c r="W9" t="s">
+        <v>43</v>
+      </c>
+      <c r="X9" t="s">
+        <v>363</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA9">
+        <v>15</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>364</v>
+      </c>
+      <c r="AD9">
+        <v>25</v>
+      </c>
+      <c r="AE9" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>134</v>
+      </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>139</v>
       </c>
@@ -4605,8 +8251,50 @@
       <c r="R10" t="s">
         <v>146</v>
       </c>
+      <c r="S10" t="s">
+        <v>368</v>
+      </c>
+      <c r="T10" t="s">
+        <v>140</v>
+      </c>
+      <c r="U10" t="s">
+        <v>44</v>
+      </c>
+      <c r="V10">
+        <v>36</v>
+      </c>
+      <c r="W10" t="s">
+        <v>141</v>
+      </c>
+      <c r="X10" t="s">
+        <v>369</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA10">
+        <v>16</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>370</v>
+      </c>
+      <c r="AD10">
+        <v>38</v>
+      </c>
+      <c r="AE10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>146</v>
+      </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>151</v>
       </c>
@@ -4661,8 +8349,50 @@
       <c r="R11" t="s">
         <v>162</v>
       </c>
+      <c r="S11" t="s">
+        <v>374</v>
+      </c>
+      <c r="T11" t="s">
+        <v>43</v>
+      </c>
+      <c r="U11" t="s">
+        <v>44</v>
+      </c>
+      <c r="V11">
+        <v>40</v>
+      </c>
+      <c r="W11" t="s">
+        <v>43</v>
+      </c>
+      <c r="X11" t="s">
+        <v>375</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA11">
+        <v>30</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>376</v>
+      </c>
+      <c r="AD11">
+        <v>52</v>
+      </c>
+      <c r="AE11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>377</v>
+      </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>167</v>
       </c>
@@ -4717,8 +8447,50 @@
       <c r="R12" t="s">
         <v>173</v>
       </c>
+      <c r="S12" t="s">
+        <v>381</v>
+      </c>
+      <c r="T12" t="s">
+        <v>382</v>
+      </c>
+      <c r="U12" t="s">
+        <v>44</v>
+      </c>
+      <c r="V12">
+        <v>26</v>
+      </c>
+      <c r="W12" t="s">
+        <v>43</v>
+      </c>
+      <c r="X12" t="s">
+        <v>383</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA12">
+        <v>21</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>384</v>
+      </c>
+      <c r="AD12">
+        <v>33</v>
+      </c>
+      <c r="AE12" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>386</v>
+      </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>178</v>
       </c>
@@ -4773,8 +8545,50 @@
       <c r="R13" t="s">
         <v>184</v>
       </c>
+      <c r="S13" t="s">
+        <v>390</v>
+      </c>
+      <c r="T13" t="s">
+        <v>391</v>
+      </c>
+      <c r="U13" t="s">
+        <v>44</v>
+      </c>
+      <c r="V13">
+        <v>27</v>
+      </c>
+      <c r="W13" t="s">
+        <v>392</v>
+      </c>
+      <c r="X13" t="s">
+        <v>393</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA13">
+        <v>11</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>394</v>
+      </c>
+      <c r="AD13">
+        <v>30</v>
+      </c>
+      <c r="AE13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>396</v>
+      </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>189</v>
       </c>
@@ -4829,8 +8643,50 @@
       <c r="R14" t="s">
         <v>196</v>
       </c>
+      <c r="S14" t="s">
+        <v>400</v>
+      </c>
+      <c r="T14" t="s">
+        <v>191</v>
+      </c>
+      <c r="U14" t="s">
+        <v>44</v>
+      </c>
+      <c r="V14">
+        <v>26</v>
+      </c>
+      <c r="W14" t="s">
+        <v>45</v>
+      </c>
+      <c r="X14" t="s">
+        <v>401</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA14">
+        <v>18</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>402</v>
+      </c>
+      <c r="AD14">
+        <v>24</v>
+      </c>
+      <c r="AE14" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>405</v>
+      </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>201</v>
       </c>
@@ -4885,8 +8741,50 @@
       <c r="R15" t="s">
         <v>206</v>
       </c>
+      <c r="S15" t="s">
+        <v>409</v>
+      </c>
+      <c r="T15" t="s">
+        <v>43</v>
+      </c>
+      <c r="U15" t="s">
+        <v>44</v>
+      </c>
+      <c r="V15">
+        <v>29</v>
+      </c>
+      <c r="W15" t="s">
+        <v>43</v>
+      </c>
+      <c r="X15" t="s">
+        <v>410</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA15">
+        <v>12</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>411</v>
+      </c>
+      <c r="AD15">
+        <v>30</v>
+      </c>
+      <c r="AE15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>414</v>
+      </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>211</v>
       </c>
@@ -4941,8 +8839,50 @@
       <c r="R16" t="s">
         <v>216</v>
       </c>
+      <c r="S16" t="s">
+        <v>418</v>
+      </c>
+      <c r="T16" t="s">
+        <v>43</v>
+      </c>
+      <c r="U16" t="s">
+        <v>44</v>
+      </c>
+      <c r="V16">
+        <v>34</v>
+      </c>
+      <c r="W16" t="s">
+        <v>43</v>
+      </c>
+      <c r="X16" t="s">
+        <v>419</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>157</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA16">
+        <v>25</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>420</v>
+      </c>
+      <c r="AD16">
+        <v>39</v>
+      </c>
+      <c r="AE16" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>421</v>
+      </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>221</v>
       </c>
@@ -4997,8 +8937,50 @@
       <c r="R17" t="s">
         <v>44</v>
       </c>
+      <c r="S17" t="s">
+        <v>425</v>
+      </c>
+      <c r="T17" t="s">
+        <v>426</v>
+      </c>
+      <c r="U17" t="s">
+        <v>44</v>
+      </c>
+      <c r="V17">
+        <v>36</v>
+      </c>
+      <c r="W17" t="s">
+        <v>43</v>
+      </c>
+      <c r="X17" t="s">
+        <v>427</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>428</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA17">
+        <v>23</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>429</v>
+      </c>
+      <c r="AD17">
+        <v>36</v>
+      </c>
+      <c r="AE17" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>432</v>
+      </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>231</v>
       </c>
@@ -5053,8 +9035,50 @@
       <c r="R18" t="s">
         <v>44</v>
       </c>
+      <c r="S18" t="s">
+        <v>436</v>
+      </c>
+      <c r="T18" t="s">
+        <v>233</v>
+      </c>
+      <c r="U18" t="s">
+        <v>44</v>
+      </c>
+      <c r="V18">
+        <v>16</v>
+      </c>
+      <c r="W18" t="s">
+        <v>43</v>
+      </c>
+      <c r="X18" t="s">
+        <v>437</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>428</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA18">
+        <v>12</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>438</v>
+      </c>
+      <c r="AD18">
+        <v>22</v>
+      </c>
+      <c r="AE18" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>377</v>
+      </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>238</v>
       </c>
@@ -5109,8 +9133,50 @@
       <c r="R19" t="s">
         <v>44</v>
       </c>
+      <c r="S19" t="s">
+        <v>443</v>
+      </c>
+      <c r="T19" t="s">
+        <v>444</v>
+      </c>
+      <c r="U19" t="s">
+        <v>44</v>
+      </c>
+      <c r="V19">
+        <v>47</v>
+      </c>
+      <c r="W19" t="s">
+        <v>119</v>
+      </c>
+      <c r="X19" t="s">
+        <v>445</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>428</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA19">
+        <v>19</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>446</v>
+      </c>
+      <c r="AD19">
+        <v>30</v>
+      </c>
+      <c r="AE19" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF19" t="s">
+        <v>449</v>
+      </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>245</v>
       </c>
@@ -5165,8 +9231,50 @@
       <c r="R20" t="s">
         <v>44</v>
       </c>
+      <c r="S20" t="s">
+        <v>453</v>
+      </c>
+      <c r="T20" t="s">
+        <v>250</v>
+      </c>
+      <c r="U20" t="s">
+        <v>44</v>
+      </c>
+      <c r="V20">
+        <v>26</v>
+      </c>
+      <c r="W20" t="s">
+        <v>43</v>
+      </c>
+      <c r="X20" t="s">
+        <v>454</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>455</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA20">
+        <v>17</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>456</v>
+      </c>
+      <c r="AD20">
+        <v>27</v>
+      </c>
+      <c r="AE20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>458</v>
+      </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>255</v>
       </c>
@@ -5221,8 +9329,50 @@
       <c r="R21" t="s">
         <v>44</v>
       </c>
+      <c r="S21" t="s">
+        <v>462</v>
+      </c>
+      <c r="T21" t="s">
+        <v>463</v>
+      </c>
+      <c r="U21" t="s">
+        <v>44</v>
+      </c>
+      <c r="V21">
+        <v>12</v>
+      </c>
+      <c r="W21" t="s">
+        <v>43</v>
+      </c>
+      <c r="X21" t="s">
+        <v>464</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>455</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA21">
+        <v>9</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>465</v>
+      </c>
+      <c r="AD21">
+        <v>15</v>
+      </c>
+      <c r="AE21" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>377</v>
+      </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>261</v>
       </c>
@@ -5277,8 +9427,50 @@
       <c r="R22" t="s">
         <v>266</v>
       </c>
+      <c r="S22" t="s">
+        <v>469</v>
+      </c>
+      <c r="T22" t="s">
+        <v>250</v>
+      </c>
+      <c r="U22" t="s">
+        <v>44</v>
+      </c>
+      <c r="V22">
+        <v>14</v>
+      </c>
+      <c r="W22" t="s">
+        <v>43</v>
+      </c>
+      <c r="X22" t="s">
+        <v>470</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>455</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA22">
+        <v>8</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>471</v>
+      </c>
+      <c r="AD22">
+        <v>12</v>
+      </c>
+      <c r="AE22" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>474</v>
+      </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>271</v>
       </c>
@@ -5333,8 +9525,50 @@
       <c r="R23" t="s">
         <v>44</v>
       </c>
+      <c r="S23" t="s">
+        <v>478</v>
+      </c>
+      <c r="T23" t="s">
+        <v>250</v>
+      </c>
+      <c r="U23" t="s">
+        <v>44</v>
+      </c>
+      <c r="V23">
+        <v>22</v>
+      </c>
+      <c r="W23" t="s">
+        <v>43</v>
+      </c>
+      <c r="X23" t="s">
+        <v>479</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>455</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA23">
+        <v>14</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>480</v>
+      </c>
+      <c r="AD23">
+        <v>21</v>
+      </c>
+      <c r="AE23" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>481</v>
+      </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>277</v>
       </c>
@@ -5389,8 +9623,50 @@
       <c r="R24" t="s">
         <v>282</v>
       </c>
+      <c r="S24" t="s">
+        <v>485</v>
+      </c>
+      <c r="T24" t="s">
+        <v>463</v>
+      </c>
+      <c r="U24" t="s">
+        <v>44</v>
+      </c>
+      <c r="V24">
+        <v>8</v>
+      </c>
+      <c r="W24" t="s">
+        <v>43</v>
+      </c>
+      <c r="X24" t="s">
+        <v>486</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>455</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA24">
+        <v>6</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>487</v>
+      </c>
+      <c r="AD24">
+        <v>9</v>
+      </c>
+      <c r="AE24" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>377</v>
+      </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>287</v>
       </c>
@@ -5445,8 +9721,50 @@
       <c r="R25" t="s">
         <v>292</v>
       </c>
+      <c r="S25" t="s">
+        <v>492</v>
+      </c>
+      <c r="T25" t="s">
+        <v>43</v>
+      </c>
+      <c r="U25" t="s">
+        <v>44</v>
+      </c>
+      <c r="V25">
+        <v>4</v>
+      </c>
+      <c r="W25" t="s">
+        <v>43</v>
+      </c>
+      <c r="X25" t="s">
+        <v>493</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>455</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA25">
+        <v>3</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>494</v>
+      </c>
+      <c r="AD25">
+        <v>6</v>
+      </c>
+      <c r="AE25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>377</v>
+      </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>297</v>
       </c>
@@ -5501,9 +9819,51 @@
       <c r="R26" t="s">
         <v>308</v>
       </c>
+      <c r="S26" t="s">
+        <v>499</v>
+      </c>
+      <c r="T26" t="s">
+        <v>500</v>
+      </c>
+      <c r="U26" t="s">
+        <v>44</v>
+      </c>
+      <c r="V26">
+        <v>25</v>
+      </c>
+      <c r="W26" t="s">
+        <v>119</v>
+      </c>
+      <c r="X26" t="s">
+        <v>501</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>304</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA26">
+        <v>7</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>48</v>
+      </c>
+      <c r="AC26" t="s">
+        <v>502</v>
+      </c>
+      <c r="AD26">
+        <v>16</v>
+      </c>
+      <c r="AE26" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF26" t="s">
+        <v>504</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R1"/>
+  <autoFilter ref="A1:AF1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Auto-collect traffic data: 2026-09-21 07:15 PM IST
</commit_message>
<xml_diff>
--- a/output/excel/Bus_vs_Metro_Data_2026-09-21_Mon.xlsx
+++ b/output/excel/Bus_vs_Metro_Data_2026-09-21_Mon.xlsx
@@ -7,14 +7,15 @@
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="1_00 PM" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="All Periods Combined" state="visible" r:id="rId7"/>
+    <sheet sheetId="4" name="7_00 PM" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="All Periods Combined" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3254" uniqueCount="747">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4300" uniqueCount="934">
   <si>
     <t>Date</t>
   </si>
@@ -2131,6 +2132,525 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/1_00_PM/MC-25/car.jpg</t>
   </si>
   <si>
+    <t>9/21/2026, 7:04:56 PM</t>
+  </si>
+  <si>
+    <t>7:00 PM</t>
+  </si>
+  <si>
+    <t>Monday (Weekday) - Evening Peak</t>
+  </si>
+  <si>
+    <t> | 50 min | 7:00 AM—7:50 AM | DN-9/1  234/1 | 7:00 AM from Dakshineswar | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 7:18 AM—7:46 AM | Blue Line | 7:18 AM from Dakshineswar | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-01/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-01/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:05:22 PM</t>
+  </si>
+  <si>
+    <t> | 51 min | 7:04 AM—7:55 AM | S-112 | 7:04 AM from Khudiram Metro | Details</t>
+  </si>
+  <si>
+    <t> | 29 min | 7:00 AM—7:29 AM | Blue Line | 7:00 AM from Shahid Khudiram | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>1.76x</t>
+  </si>
+  <si>
+    <t>43.1% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-02/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-02/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:05:47 PM</t>
+  </si>
+  <si>
+    <t> | 12 min | 7:07 AM—7:19 AM | S-10 | 7:07 AM from Dumdum Station | Details</t>
+  </si>
+  <si>
+    <t> | 8 min | 7:01 AM—7:09 AM | Blue Line | 7:01 AM from Shyambazar | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>1.50x</t>
+  </si>
+  <si>
+    <t>33.3% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-03/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-03/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:06:14 PM</t>
+  </si>
+  <si>
+    <t> | 18 min | 7:02 AM—7:20 AM | 47B | 7:02 AM from Shyambazar | Details</t>
+  </si>
+  <si>
+    <t> | 11 min | 7:00 AM—7:11 AM | Blue Line | 7:00 AM from Shyambazar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-04/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-04/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:06:41 PM</t>
+  </si>
+  <si>
+    <t> | 18 min | 7:04 AM—7:22 AM | M-7B | 7:04 AM from S.P. Mukherjee Road / R.B. Avenue Crossing | Details</t>
+  </si>
+  <si>
+    <t> | 11 min | 7:09 AM—7:20 AM | Blue Line | 7:09 AM from Kalighat | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-05/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-05/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:07:08 PM</t>
+  </si>
+  <si>
+    <t> | 24 min | 7:00 AM—7:24 AM | DN-9/1 | 7:00 AM from Dakshineswar | Details</t>
+  </si>
+  <si>
+    <t> | 12 min | 7:18 AM—7:30 AM | Blue Line | 7:18 AM from Dakshineswar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-06/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:07:35 PM</t>
+  </si>
+  <si>
+    <t> | 27 min | 7:11 AM—7:38 AM | 12C/1B | 7:11 AM from Esplanade Metro | Details</t>
+  </si>
+  <si>
+    <t> | 18 min | 7:11 AM—7:29 AM | Blue Line | 7:11 AM from Esplanade | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-07/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-07/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:08:02 PM</t>
+  </si>
+  <si>
+    <t> | 22 min | 7:09 AM—7:31 AM | S-112 | 7:09 AM from Tollygunge Tram Depot | Details</t>
+  </si>
+  <si>
+    <t> | 15 min | 7:01 AM—7:16 AM | Blue Line | 7:01 AM from Mahanayak Uttam Kumar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-08/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-08/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:08:28 PM</t>
+  </si>
+  <si>
+    <t> | 30 min | 7:07 AM—7:37 AM | S-10 | 7:07 AM from Dumdum Station | Details</t>
+  </si>
+  <si>
+    <t> | 16 min | 7:09 AM—7:25 AM | Blue Line | 7:09 AM from Dumdum | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t>14 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.88x</t>
+  </si>
+  <si>
+    <t>46.7% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-09/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-09/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:08:54 PM</t>
+  </si>
+  <si>
+    <t> | 40 min | 7:00 AM—7:40 AM | 215A/1 | 7:00 AM from Howrah Station | Details</t>
+  </si>
+  <si>
+    <t> | 30 min | 7:02 AM—7:32 AM | Green Line | 7:02 AM from Howrah | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-10/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-10/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:09:20 PM</t>
+  </si>
+  <si>
+    <t> | 25 min | 7:04 AM—7:29 AM | S-12N | 7:04 AM from Sealdah - B.R. Singh Hospital | Details</t>
+  </si>
+  <si>
+    <t> | 21 min | 7:11 AM—7:32 AM | Green Line | 7:11 AM from Sealdah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-11/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-11/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:09:45 PM</t>
+  </si>
+  <si>
+    <t> | 17 min | 7:00 AM—7:17 AM | 28 | 7:00 AM from Howrah Maidan | Details</t>
+  </si>
+  <si>
+    <t> | 11 min | 7:00 AM—7:11 AM | Green Line | 7:00 AM from Howrah Maidan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-12/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-12/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:10:13 PM</t>
+  </si>
+  <si>
+    <t>S-21</t>
+  </si>
+  <si>
+    <t> | 25 min | 7:04 AM—7:29 AM | S-21  S-12N | 7:04 AM from Phoolbagan | Details</t>
+  </si>
+  <si>
+    <t> | 18 min | 7:14 AM—7:32 AM | Green Line | 7:14 AM from Phoolbagan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>1.39x</t>
+  </si>
+  <si>
+    <t>28.0% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-13/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-13/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:10:39 PM</t>
+  </si>
+  <si>
+    <t> | 23 min | 7:07 AM—7:30 AM | 44   | 7:07 AM from Howrah Station |  4 min | Details</t>
+  </si>
+  <si>
+    <t> | 12 min | 7:02 AM—7:14 AM | Green Line | 7:02 AM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-14/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-14/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:11:06 PM</t>
+  </si>
+  <si>
+    <t> | 34 min | 7:25 AM—7:59 AM | S-12N | 7:25 AM from Esplanade Metro | Details</t>
+  </si>
+  <si>
+    <t> | 25 min | 7:07 AM—7:32 AM | Green Line | 7:07 AM from Esplanade | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-15/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-15/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:11:32 PM</t>
+  </si>
+  <si>
+    <t> | 36 min | 7:03 AM—7:39 AM | AS-3 | 7:03 AM from Dhalai Bridge | Details</t>
+  </si>
+  <si>
+    <t>22.2% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-16/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-16/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:11:58 PM</t>
+  </si>
+  <si>
+    <t>EB-3</t>
+  </si>
+  <si>
+    <t> | 16 min | 7:00 AM—7:16 AM | EB-3 | 7:00 AM from Ruby | Details</t>
+  </si>
+  <si>
+    <t> | 17 min | 7:51 AM—8:08 AM | Orange Line | 7:51 AM from Hemanta Mukhopadhyay | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>1 min (Bus Faster)</t>
+  </si>
+  <si>
+    <t>0.94x</t>
+  </si>
+  <si>
+    <t>5.9% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-17/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-17/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:12:25 PM</t>
+  </si>
+  <si>
+    <t> | 47 min | 7:02 AM—7:49 AM |   C26A</t>
+  </si>
+  <si>
+    <t>51.1% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-18/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-18/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:12:51 PM</t>
+  </si>
+  <si>
+    <t> | 26 min | 7:01 AM—7:27 AM | S-131 | 7:01 AM from Diamond Park | Details</t>
+  </si>
+  <si>
+    <t> | 17 min | 7:03 AM—7:20 AM | Purple Line | 7:03 AM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-19/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-19/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:13:16 PM</t>
+  </si>
+  <si>
+    <t> | 12 min | 7:01 AM—7:13 AM | S-21 Minibus | 7:01 AM from Behala Chowrasta | Details</t>
+  </si>
+  <si>
+    <t> | 9 min | 7:11 AM—7:20 AM | Purple Line | 7:11 AM from Behala Chowrasta | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-20/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-20/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:13:43 PM</t>
+  </si>
+  <si>
+    <t> | 14 min | 7:01 AM—7:15 AM | S-131 | 7:01 AM from Diamond Park | Details</t>
+  </si>
+  <si>
+    <t> | 8 min | 7:03 AM—7:11 AM | Purple Line | 7:03 AM from Joka | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-21/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-21/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:14:09 PM</t>
+  </si>
+  <si>
+    <t> | 22 min | 7:01 AM—7:23 AM | S-131 | 7:01 AM from Diamond Park | Details</t>
+  </si>
+  <si>
+    <t> | 14 min | 7:03 AM—7:17 AM | Purple Line | 7:03 AM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-22/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-22/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:14:35 PM</t>
+  </si>
+  <si>
+    <t> | 7 min | 7:01 AM—7:08 AM | S-21 Minibus | 7:01 AM from Behala Chowrasta | Details</t>
+  </si>
+  <si>
+    <t> | 6 min | 7:11 AM—7:17 AM | Purple Line | 7:11 AM from Behala Chowrasta | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>1.17x</t>
+  </si>
+  <si>
+    <t>14.3% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-23/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-23/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:15:00 PM</t>
+  </si>
+  <si>
+    <t> | 4 min | 7:01 AM—7:05 AM | S-12D | 7:01 AM from Pathak Para | Details</t>
+  </si>
+  <si>
+    <t> | 3 min | 7:17 AM—7:20 AM | Purple Line | 7:17 AM from Taratala | ₹5.00 | Details</t>
+  </si>
+  <si>
+    <t>Tie</t>
+  </si>
+  <si>
+    <t>0%</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-24/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-24/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-24/car.jpg</t>
+  </si>
+  <si>
+    <t>9/21/2026, 7:15:27 PM</t>
+  </si>
+  <si>
+    <t>30D, 79B</t>
+  </si>
+  <si>
+    <t> | 26 min | 7:10 AM—7:36 AM | 30D  79B | 7:10 AM from Dumdum Cantonment Station |  1 min | Details</t>
+  </si>
+  <si>
+    <t> | 9 min | 7:24 AM—7:33 AM | Yellow Line | 7:24 AM from Dum Dum Cantonment | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>2.89x</t>
+  </si>
+  <si>
+    <t>65.4% (vs Bus)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-25/bus.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-25/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-21/7_00_PM/MC-25/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -2255,6 +2775,48 @@
   </si>
   <si>
     <t>1:00 PM Savings (%)</t>
+  </si>
+  <si>
+    <t>7:00 PM Scraped At</t>
+  </si>
+  <si>
+    <t>7:00 PM Actual Bus</t>
+  </si>
+  <si>
+    <t>7:00 PM Bus Walk</t>
+  </si>
+  <si>
+    <t>7:00 PM Bus (min)</t>
+  </si>
+  <si>
+    <t>7:00 PM Bus Route</t>
+  </si>
+  <si>
+    <t>7:00 PM Bus Raw Details</t>
+  </si>
+  <si>
+    <t>7:00 PM Actual Metro</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Walk</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro (min)</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Route</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>7:00 PM Car (min)</t>
+  </si>
+  <si>
+    <t>7:00 PM Faster Mode</t>
+  </si>
+  <si>
+    <t>7:00 PM Savings (%)</t>
   </si>
 </sst>
 </file>
@@ -10587,10 +11149,2647 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AT26"/>
+  <dimension ref="A1:AF26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:46" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>705</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" t="s">
+        <v>706</v>
+      </c>
+      <c r="K2" t="s">
+        <v>707</v>
+      </c>
+      <c r="L2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M2" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2">
+        <v>50</v>
+      </c>
+      <c r="O2" t="s">
+        <v>45</v>
+      </c>
+      <c r="P2" t="s">
+        <v>708</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>47</v>
+      </c>
+      <c r="R2" t="s">
+        <v>44</v>
+      </c>
+      <c r="S2">
+        <v>28</v>
+      </c>
+      <c r="T2" t="s">
+        <v>48</v>
+      </c>
+      <c r="U2" t="s">
+        <v>709</v>
+      </c>
+      <c r="V2">
+        <v>53</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="X2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>710</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>711</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>713</v>
+      </c>
+      <c r="D3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J3" t="s">
+        <v>706</v>
+      </c>
+      <c r="K3" t="s">
+        <v>707</v>
+      </c>
+      <c r="L3" t="s">
+        <v>61</v>
+      </c>
+      <c r="M3" t="s">
+        <v>44</v>
+      </c>
+      <c r="N3">
+        <v>51</v>
+      </c>
+      <c r="O3" t="s">
+        <v>43</v>
+      </c>
+      <c r="P3" t="s">
+        <v>714</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>47</v>
+      </c>
+      <c r="R3" t="s">
+        <v>44</v>
+      </c>
+      <c r="S3">
+        <v>29</v>
+      </c>
+      <c r="T3" t="s">
+        <v>48</v>
+      </c>
+      <c r="U3" t="s">
+        <v>715</v>
+      </c>
+      <c r="V3">
+        <v>65</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="X3" t="s">
+        <v>716</v>
+      </c>
+      <c r="Y3" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>717</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>718</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>719</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
+        <v>721</v>
+      </c>
+      <c r="D4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J4" t="s">
+        <v>706</v>
+      </c>
+      <c r="K4" t="s">
+        <v>707</v>
+      </c>
+      <c r="L4" t="s">
+        <v>336</v>
+      </c>
+      <c r="M4" t="s">
+        <v>44</v>
+      </c>
+      <c r="N4">
+        <v>12</v>
+      </c>
+      <c r="O4" t="s">
+        <v>43</v>
+      </c>
+      <c r="P4" t="s">
+        <v>722</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>47</v>
+      </c>
+      <c r="R4" t="s">
+        <v>44</v>
+      </c>
+      <c r="S4">
+        <v>8</v>
+      </c>
+      <c r="T4" t="s">
+        <v>48</v>
+      </c>
+      <c r="U4" t="s">
+        <v>723</v>
+      </c>
+      <c r="V4">
+        <v>17</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="X4" t="s">
+        <v>724</v>
+      </c>
+      <c r="Y4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>725</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>726</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>727</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>729</v>
+      </c>
+      <c r="D5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H5" t="s">
+        <v>74</v>
+      </c>
+      <c r="I5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" t="s">
+        <v>706</v>
+      </c>
+      <c r="K5" t="s">
+        <v>707</v>
+      </c>
+      <c r="L5" t="s">
+        <v>87</v>
+      </c>
+      <c r="M5" t="s">
+        <v>44</v>
+      </c>
+      <c r="N5">
+        <v>18</v>
+      </c>
+      <c r="O5" t="s">
+        <v>43</v>
+      </c>
+      <c r="P5" t="s">
+        <v>730</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>47</v>
+      </c>
+      <c r="R5" t="s">
+        <v>44</v>
+      </c>
+      <c r="S5">
+        <v>11</v>
+      </c>
+      <c r="T5" t="s">
+        <v>48</v>
+      </c>
+      <c r="U5" t="s">
+        <v>731</v>
+      </c>
+      <c r="V5">
+        <v>33</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="X5" t="s">
+        <v>91</v>
+      </c>
+      <c r="Y5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>92</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>732</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>733</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
+        <v>735</v>
+      </c>
+      <c r="D6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" t="s">
+        <v>72</v>
+      </c>
+      <c r="H6" t="s">
+        <v>98</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J6" t="s">
+        <v>706</v>
+      </c>
+      <c r="K6" t="s">
+        <v>707</v>
+      </c>
+      <c r="L6" t="s">
+        <v>43</v>
+      </c>
+      <c r="M6" t="s">
+        <v>44</v>
+      </c>
+      <c r="N6">
+        <v>18</v>
+      </c>
+      <c r="O6" t="s">
+        <v>43</v>
+      </c>
+      <c r="P6" t="s">
+        <v>736</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>47</v>
+      </c>
+      <c r="R6" t="s">
+        <v>44</v>
+      </c>
+      <c r="S6">
+        <v>11</v>
+      </c>
+      <c r="T6" t="s">
+        <v>48</v>
+      </c>
+      <c r="U6" t="s">
+        <v>737</v>
+      </c>
+      <c r="V6">
+        <v>22</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="X6" t="s">
+        <v>91</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>92</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>738</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>739</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
+        <v>741</v>
+      </c>
+      <c r="D7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
+        <v>73</v>
+      </c>
+      <c r="J7" t="s">
+        <v>706</v>
+      </c>
+      <c r="K7" t="s">
+        <v>707</v>
+      </c>
+      <c r="L7" t="s">
+        <v>43</v>
+      </c>
+      <c r="M7" t="s">
+        <v>44</v>
+      </c>
+      <c r="N7">
+        <v>24</v>
+      </c>
+      <c r="O7" t="s">
+        <v>43</v>
+      </c>
+      <c r="P7" t="s">
+        <v>742</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>47</v>
+      </c>
+      <c r="R7" t="s">
+        <v>44</v>
+      </c>
+      <c r="S7">
+        <v>12</v>
+      </c>
+      <c r="T7" t="s">
+        <v>48</v>
+      </c>
+      <c r="U7" t="s">
+        <v>743</v>
+      </c>
+      <c r="V7">
+        <v>26</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="X7" t="s">
+        <v>110</v>
+      </c>
+      <c r="Y7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>744</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>745</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
+        <v>747</v>
+      </c>
+      <c r="D8" t="s">
+        <v>116</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>72</v>
+      </c>
+      <c r="H8" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" t="s">
+        <v>117</v>
+      </c>
+      <c r="J8" t="s">
+        <v>706</v>
+      </c>
+      <c r="K8" t="s">
+        <v>707</v>
+      </c>
+      <c r="L8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M8" t="s">
+        <v>44</v>
+      </c>
+      <c r="N8">
+        <v>27</v>
+      </c>
+      <c r="O8" t="s">
+        <v>43</v>
+      </c>
+      <c r="P8" t="s">
+        <v>748</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>47</v>
+      </c>
+      <c r="R8" t="s">
+        <v>44</v>
+      </c>
+      <c r="S8">
+        <v>18</v>
+      </c>
+      <c r="T8" t="s">
+        <v>48</v>
+      </c>
+      <c r="U8" t="s">
+        <v>749</v>
+      </c>
+      <c r="V8">
+        <v>37</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="X8" t="s">
+        <v>724</v>
+      </c>
+      <c r="Y8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>725</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>750</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>751</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" t="s">
+        <v>753</v>
+      </c>
+      <c r="D9" t="s">
+        <v>129</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" t="s">
+        <v>72</v>
+      </c>
+      <c r="H9" t="s">
+        <v>117</v>
+      </c>
+      <c r="I9" t="s">
+        <v>130</v>
+      </c>
+      <c r="J9" t="s">
+        <v>706</v>
+      </c>
+      <c r="K9" t="s">
+        <v>707</v>
+      </c>
+      <c r="L9" t="s">
+        <v>61</v>
+      </c>
+      <c r="M9" t="s">
+        <v>44</v>
+      </c>
+      <c r="N9">
+        <v>22</v>
+      </c>
+      <c r="O9" t="s">
+        <v>43</v>
+      </c>
+      <c r="P9" t="s">
+        <v>754</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>47</v>
+      </c>
+      <c r="R9" t="s">
+        <v>44</v>
+      </c>
+      <c r="S9">
+        <v>15</v>
+      </c>
+      <c r="T9" t="s">
+        <v>48</v>
+      </c>
+      <c r="U9" t="s">
+        <v>755</v>
+      </c>
+      <c r="V9">
+        <v>33</v>
+      </c>
+      <c r="W9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="X9" t="s">
+        <v>133</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>134</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>756</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>757</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>759</v>
+      </c>
+      <c r="D10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" t="s">
+        <v>72</v>
+      </c>
+      <c r="H10" t="s">
+        <v>73</v>
+      </c>
+      <c r="I10" t="s">
+        <v>40</v>
+      </c>
+      <c r="J10" t="s">
+        <v>706</v>
+      </c>
+      <c r="K10" t="s">
+        <v>707</v>
+      </c>
+      <c r="L10" t="s">
+        <v>336</v>
+      </c>
+      <c r="M10" t="s">
+        <v>44</v>
+      </c>
+      <c r="N10">
+        <v>30</v>
+      </c>
+      <c r="O10" t="s">
+        <v>43</v>
+      </c>
+      <c r="P10" t="s">
+        <v>760</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>47</v>
+      </c>
+      <c r="R10" t="s">
+        <v>44</v>
+      </c>
+      <c r="S10">
+        <v>16</v>
+      </c>
+      <c r="T10" t="s">
+        <v>48</v>
+      </c>
+      <c r="U10" t="s">
+        <v>761</v>
+      </c>
+      <c r="V10">
+        <v>47</v>
+      </c>
+      <c r="W10" s="2" t="s">
+        <v>762</v>
+      </c>
+      <c r="X10" t="s">
+        <v>763</v>
+      </c>
+      <c r="Y10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>764</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>765</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>766</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" t="s">
+        <v>768</v>
+      </c>
+      <c r="D11" t="s">
+        <v>151</v>
+      </c>
+      <c r="E11" t="s">
+        <v>152</v>
+      </c>
+      <c r="F11" t="s">
+        <v>153</v>
+      </c>
+      <c r="G11" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" t="s">
+        <v>154</v>
+      </c>
+      <c r="I11" t="s">
+        <v>155</v>
+      </c>
+      <c r="J11" t="s">
+        <v>706</v>
+      </c>
+      <c r="K11" t="s">
+        <v>707</v>
+      </c>
+      <c r="L11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M11" t="s">
+        <v>44</v>
+      </c>
+      <c r="N11">
+        <v>40</v>
+      </c>
+      <c r="O11" t="s">
+        <v>43</v>
+      </c>
+      <c r="P11" t="s">
+        <v>769</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>157</v>
+      </c>
+      <c r="R11" t="s">
+        <v>44</v>
+      </c>
+      <c r="S11">
+        <v>30</v>
+      </c>
+      <c r="T11" t="s">
+        <v>48</v>
+      </c>
+      <c r="U11" t="s">
+        <v>770</v>
+      </c>
+      <c r="V11">
+        <v>63</v>
+      </c>
+      <c r="W11" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="X11" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>377</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>771</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>772</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s">
+        <v>774</v>
+      </c>
+      <c r="D12" t="s">
+        <v>167</v>
+      </c>
+      <c r="E12" t="s">
+        <v>152</v>
+      </c>
+      <c r="F12" t="s">
+        <v>153</v>
+      </c>
+      <c r="G12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H12" t="s">
+        <v>168</v>
+      </c>
+      <c r="I12" t="s">
+        <v>155</v>
+      </c>
+      <c r="J12" t="s">
+        <v>706</v>
+      </c>
+      <c r="K12" t="s">
+        <v>707</v>
+      </c>
+      <c r="L12" t="s">
+        <v>43</v>
+      </c>
+      <c r="M12" t="s">
+        <v>44</v>
+      </c>
+      <c r="N12">
+        <v>25</v>
+      </c>
+      <c r="O12" t="s">
+        <v>43</v>
+      </c>
+      <c r="P12" t="s">
+        <v>775</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>157</v>
+      </c>
+      <c r="R12" t="s">
+        <v>44</v>
+      </c>
+      <c r="S12">
+        <v>21</v>
+      </c>
+      <c r="T12" t="s">
+        <v>48</v>
+      </c>
+      <c r="U12" t="s">
+        <v>776</v>
+      </c>
+      <c r="V12">
+        <v>31</v>
+      </c>
+      <c r="W12" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="X12" t="s">
+        <v>595</v>
+      </c>
+      <c r="Y12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>596</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>777</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>778</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" t="s">
+        <v>780</v>
+      </c>
+      <c r="D13" t="s">
+        <v>178</v>
+      </c>
+      <c r="E13" t="s">
+        <v>152</v>
+      </c>
+      <c r="F13" t="s">
+        <v>179</v>
+      </c>
+      <c r="G13" t="s">
+        <v>72</v>
+      </c>
+      <c r="H13" t="s">
+        <v>154</v>
+      </c>
+      <c r="I13" t="s">
+        <v>168</v>
+      </c>
+      <c r="J13" t="s">
+        <v>706</v>
+      </c>
+      <c r="K13" t="s">
+        <v>707</v>
+      </c>
+      <c r="L13" t="s">
+        <v>180</v>
+      </c>
+      <c r="M13" t="s">
+        <v>44</v>
+      </c>
+      <c r="N13">
+        <v>17</v>
+      </c>
+      <c r="O13" t="s">
+        <v>43</v>
+      </c>
+      <c r="P13" t="s">
+        <v>781</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>157</v>
+      </c>
+      <c r="R13" t="s">
+        <v>44</v>
+      </c>
+      <c r="S13">
+        <v>11</v>
+      </c>
+      <c r="T13" t="s">
+        <v>48</v>
+      </c>
+      <c r="U13" t="s">
+        <v>782</v>
+      </c>
+      <c r="V13">
+        <v>37</v>
+      </c>
+      <c r="W13" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="X13" t="s">
+        <v>603</v>
+      </c>
+      <c r="Y13" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>604</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>783</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>784</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
+        <v>786</v>
+      </c>
+      <c r="D14" t="s">
+        <v>189</v>
+      </c>
+      <c r="E14" t="s">
+        <v>152</v>
+      </c>
+      <c r="F14" t="s">
+        <v>179</v>
+      </c>
+      <c r="G14" t="s">
+        <v>72</v>
+      </c>
+      <c r="H14" t="s">
+        <v>190</v>
+      </c>
+      <c r="I14" t="s">
+        <v>155</v>
+      </c>
+      <c r="J14" t="s">
+        <v>706</v>
+      </c>
+      <c r="K14" t="s">
+        <v>707</v>
+      </c>
+      <c r="L14" t="s">
+        <v>787</v>
+      </c>
+      <c r="M14" t="s">
+        <v>44</v>
+      </c>
+      <c r="N14">
+        <v>25</v>
+      </c>
+      <c r="O14" t="s">
+        <v>45</v>
+      </c>
+      <c r="P14" t="s">
+        <v>788</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>157</v>
+      </c>
+      <c r="R14" t="s">
+        <v>44</v>
+      </c>
+      <c r="S14">
+        <v>18</v>
+      </c>
+      <c r="T14" t="s">
+        <v>48</v>
+      </c>
+      <c r="U14" t="s">
+        <v>789</v>
+      </c>
+      <c r="V14">
+        <v>24</v>
+      </c>
+      <c r="W14" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="X14" t="s">
+        <v>790</v>
+      </c>
+      <c r="Y14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>791</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>792</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>793</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>795</v>
+      </c>
+      <c r="D15" t="s">
+        <v>201</v>
+      </c>
+      <c r="E15" t="s">
+        <v>152</v>
+      </c>
+      <c r="F15" t="s">
+        <v>153</v>
+      </c>
+      <c r="G15" t="s">
+        <v>72</v>
+      </c>
+      <c r="H15" t="s">
+        <v>154</v>
+      </c>
+      <c r="I15" t="s">
+        <v>190</v>
+      </c>
+      <c r="J15" t="s">
+        <v>706</v>
+      </c>
+      <c r="K15" t="s">
+        <v>707</v>
+      </c>
+      <c r="L15" t="s">
+        <v>617</v>
+      </c>
+      <c r="M15" t="s">
+        <v>44</v>
+      </c>
+      <c r="N15">
+        <v>23</v>
+      </c>
+      <c r="O15" t="s">
+        <v>141</v>
+      </c>
+      <c r="P15" t="s">
+        <v>796</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>157</v>
+      </c>
+      <c r="R15" t="s">
+        <v>44</v>
+      </c>
+      <c r="S15">
+        <v>12</v>
+      </c>
+      <c r="T15" t="s">
+        <v>48</v>
+      </c>
+      <c r="U15" t="s">
+        <v>797</v>
+      </c>
+      <c r="V15">
+        <v>45</v>
+      </c>
+      <c r="W15" s="2" t="s">
+        <v>620</v>
+      </c>
+      <c r="X15" t="s">
+        <v>621</v>
+      </c>
+      <c r="Y15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>622</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>798</v>
+      </c>
+      <c r="AE15" t="s">
+        <v>799</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s">
+        <v>801</v>
+      </c>
+      <c r="D16" t="s">
+        <v>211</v>
+      </c>
+      <c r="E16" t="s">
+        <v>152</v>
+      </c>
+      <c r="F16" t="s">
+        <v>153</v>
+      </c>
+      <c r="G16" t="s">
+        <v>72</v>
+      </c>
+      <c r="H16" t="s">
+        <v>40</v>
+      </c>
+      <c r="I16" t="s">
+        <v>155</v>
+      </c>
+      <c r="J16" t="s">
+        <v>706</v>
+      </c>
+      <c r="K16" t="s">
+        <v>707</v>
+      </c>
+      <c r="L16" t="s">
+        <v>43</v>
+      </c>
+      <c r="M16" t="s">
+        <v>44</v>
+      </c>
+      <c r="N16">
+        <v>34</v>
+      </c>
+      <c r="O16" t="s">
+        <v>43</v>
+      </c>
+      <c r="P16" t="s">
+        <v>802</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>157</v>
+      </c>
+      <c r="R16" t="s">
+        <v>44</v>
+      </c>
+      <c r="S16">
+        <v>25</v>
+      </c>
+      <c r="T16" t="s">
+        <v>48</v>
+      </c>
+      <c r="U16" t="s">
+        <v>803</v>
+      </c>
+      <c r="V16">
+        <v>49</v>
+      </c>
+      <c r="W16" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="X16" t="s">
+        <v>215</v>
+      </c>
+      <c r="Y16" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>421</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>804</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>805</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" t="s">
+        <v>807</v>
+      </c>
+      <c r="D17" t="s">
+        <v>221</v>
+      </c>
+      <c r="E17" t="s">
+        <v>222</v>
+      </c>
+      <c r="F17" t="s">
+        <v>223</v>
+      </c>
+      <c r="G17" t="s">
+        <v>38</v>
+      </c>
+      <c r="H17" t="s">
+        <v>130</v>
+      </c>
+      <c r="I17" t="s">
+        <v>224</v>
+      </c>
+      <c r="J17" t="s">
+        <v>706</v>
+      </c>
+      <c r="K17" t="s">
+        <v>707</v>
+      </c>
+      <c r="L17" t="s">
+        <v>426</v>
+      </c>
+      <c r="M17" t="s">
+        <v>44</v>
+      </c>
+      <c r="N17">
+        <v>36</v>
+      </c>
+      <c r="O17" t="s">
+        <v>43</v>
+      </c>
+      <c r="P17" t="s">
+        <v>808</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>428</v>
+      </c>
+      <c r="R17" t="s">
+        <v>44</v>
+      </c>
+      <c r="S17">
+        <v>28</v>
+      </c>
+      <c r="T17" t="s">
+        <v>48</v>
+      </c>
+      <c r="U17" t="s">
+        <v>634</v>
+      </c>
+      <c r="V17">
+        <v>42</v>
+      </c>
+      <c r="W17" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="X17" t="s">
+        <v>569</v>
+      </c>
+      <c r="Y17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>809</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>810</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>811</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="s">
+        <v>813</v>
+      </c>
+      <c r="D18" t="s">
+        <v>231</v>
+      </c>
+      <c r="E18" t="s">
+        <v>222</v>
+      </c>
+      <c r="F18" t="s">
+        <v>179</v>
+      </c>
+      <c r="G18" t="s">
+        <v>72</v>
+      </c>
+      <c r="H18" t="s">
+        <v>232</v>
+      </c>
+      <c r="I18" t="s">
+        <v>224</v>
+      </c>
+      <c r="J18" t="s">
+        <v>706</v>
+      </c>
+      <c r="K18" t="s">
+        <v>707</v>
+      </c>
+      <c r="L18" t="s">
+        <v>814</v>
+      </c>
+      <c r="M18" t="s">
+        <v>44</v>
+      </c>
+      <c r="N18">
+        <v>16</v>
+      </c>
+      <c r="O18" t="s">
+        <v>43</v>
+      </c>
+      <c r="P18" t="s">
+        <v>815</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>428</v>
+      </c>
+      <c r="R18" t="s">
+        <v>44</v>
+      </c>
+      <c r="S18">
+        <v>17</v>
+      </c>
+      <c r="T18" t="s">
+        <v>48</v>
+      </c>
+      <c r="U18" t="s">
+        <v>816</v>
+      </c>
+      <c r="V18">
+        <v>27</v>
+      </c>
+      <c r="W18" s="4" t="s">
+        <v>817</v>
+      </c>
+      <c r="X18" t="s">
+        <v>818</v>
+      </c>
+      <c r="Y18" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>819</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>820</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>821</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" t="s">
+        <v>823</v>
+      </c>
+      <c r="D19" t="s">
+        <v>238</v>
+      </c>
+      <c r="E19" t="s">
+        <v>222</v>
+      </c>
+      <c r="F19" t="s">
+        <v>223</v>
+      </c>
+      <c r="G19" t="s">
+        <v>72</v>
+      </c>
+      <c r="H19" t="s">
+        <v>130</v>
+      </c>
+      <c r="I19" t="s">
+        <v>239</v>
+      </c>
+      <c r="J19" t="s">
+        <v>706</v>
+      </c>
+      <c r="K19" t="s">
+        <v>707</v>
+      </c>
+      <c r="L19" t="s">
+        <v>444</v>
+      </c>
+      <c r="M19" t="s">
+        <v>44</v>
+      </c>
+      <c r="N19">
+        <v>47</v>
+      </c>
+      <c r="O19" t="s">
+        <v>119</v>
+      </c>
+      <c r="P19" t="s">
+        <v>824</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>428</v>
+      </c>
+      <c r="R19" t="s">
+        <v>44</v>
+      </c>
+      <c r="S19">
+        <v>23</v>
+      </c>
+      <c r="T19" t="s">
+        <v>48</v>
+      </c>
+      <c r="U19" t="s">
+        <v>651</v>
+      </c>
+      <c r="V19">
+        <v>40</v>
+      </c>
+      <c r="W19" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="X19" t="s">
+        <v>653</v>
+      </c>
+      <c r="Y19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>825</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>826</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>827</v>
+      </c>
+      <c r="AF19" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" t="s">
+        <v>829</v>
+      </c>
+      <c r="D20" t="s">
+        <v>245</v>
+      </c>
+      <c r="E20" t="s">
+        <v>246</v>
+      </c>
+      <c r="F20" t="s">
+        <v>247</v>
+      </c>
+      <c r="G20" t="s">
+        <v>38</v>
+      </c>
+      <c r="H20" t="s">
+        <v>248</v>
+      </c>
+      <c r="I20" t="s">
+        <v>249</v>
+      </c>
+      <c r="J20" t="s">
+        <v>706</v>
+      </c>
+      <c r="K20" t="s">
+        <v>707</v>
+      </c>
+      <c r="L20" t="s">
+        <v>250</v>
+      </c>
+      <c r="M20" t="s">
+        <v>44</v>
+      </c>
+      <c r="N20">
+        <v>26</v>
+      </c>
+      <c r="O20" t="s">
+        <v>43</v>
+      </c>
+      <c r="P20" t="s">
+        <v>830</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>455</v>
+      </c>
+      <c r="R20" t="s">
+        <v>44</v>
+      </c>
+      <c r="S20">
+        <v>17</v>
+      </c>
+      <c r="T20" t="s">
+        <v>48</v>
+      </c>
+      <c r="U20" t="s">
+        <v>831</v>
+      </c>
+      <c r="V20">
+        <v>25</v>
+      </c>
+      <c r="W20" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="X20" t="s">
+        <v>457</v>
+      </c>
+      <c r="Y20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>458</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>832</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>833</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" t="s">
+        <v>835</v>
+      </c>
+      <c r="D21" t="s">
+        <v>255</v>
+      </c>
+      <c r="E21" t="s">
+        <v>246</v>
+      </c>
+      <c r="F21" t="s">
+        <v>179</v>
+      </c>
+      <c r="G21" t="s">
+        <v>72</v>
+      </c>
+      <c r="H21" t="s">
+        <v>256</v>
+      </c>
+      <c r="I21" t="s">
+        <v>249</v>
+      </c>
+      <c r="J21" t="s">
+        <v>706</v>
+      </c>
+      <c r="K21" t="s">
+        <v>707</v>
+      </c>
+      <c r="L21" t="s">
+        <v>43</v>
+      </c>
+      <c r="M21" t="s">
+        <v>44</v>
+      </c>
+      <c r="N21">
+        <v>12</v>
+      </c>
+      <c r="O21" t="s">
+        <v>43</v>
+      </c>
+      <c r="P21" t="s">
+        <v>836</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>455</v>
+      </c>
+      <c r="R21" t="s">
+        <v>44</v>
+      </c>
+      <c r="S21">
+        <v>9</v>
+      </c>
+      <c r="T21" t="s">
+        <v>48</v>
+      </c>
+      <c r="U21" t="s">
+        <v>837</v>
+      </c>
+      <c r="V21">
+        <v>11</v>
+      </c>
+      <c r="W21" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="X21" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y21" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>377</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>838</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>839</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" t="s">
+        <v>841</v>
+      </c>
+      <c r="D22" t="s">
+        <v>261</v>
+      </c>
+      <c r="E22" t="s">
+        <v>246</v>
+      </c>
+      <c r="F22" t="s">
+        <v>179</v>
+      </c>
+      <c r="G22" t="s">
+        <v>72</v>
+      </c>
+      <c r="H22" t="s">
+        <v>248</v>
+      </c>
+      <c r="I22" t="s">
+        <v>256</v>
+      </c>
+      <c r="J22" t="s">
+        <v>706</v>
+      </c>
+      <c r="K22" t="s">
+        <v>707</v>
+      </c>
+      <c r="L22" t="s">
+        <v>250</v>
+      </c>
+      <c r="M22" t="s">
+        <v>44</v>
+      </c>
+      <c r="N22">
+        <v>14</v>
+      </c>
+      <c r="O22" t="s">
+        <v>43</v>
+      </c>
+      <c r="P22" t="s">
+        <v>842</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>455</v>
+      </c>
+      <c r="R22" t="s">
+        <v>44</v>
+      </c>
+      <c r="S22">
+        <v>8</v>
+      </c>
+      <c r="T22" t="s">
+        <v>48</v>
+      </c>
+      <c r="U22" t="s">
+        <v>843</v>
+      </c>
+      <c r="V22">
+        <v>13</v>
+      </c>
+      <c r="W22" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="X22" t="s">
+        <v>473</v>
+      </c>
+      <c r="Y22" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>474</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>844</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>845</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" t="s">
+        <v>847</v>
+      </c>
+      <c r="D23" t="s">
+        <v>271</v>
+      </c>
+      <c r="E23" t="s">
+        <v>246</v>
+      </c>
+      <c r="F23" t="s">
+        <v>247</v>
+      </c>
+      <c r="G23" t="s">
+        <v>72</v>
+      </c>
+      <c r="H23" t="s">
+        <v>248</v>
+      </c>
+      <c r="I23" t="s">
+        <v>272</v>
+      </c>
+      <c r="J23" t="s">
+        <v>706</v>
+      </c>
+      <c r="K23" t="s">
+        <v>707</v>
+      </c>
+      <c r="L23" t="s">
+        <v>250</v>
+      </c>
+      <c r="M23" t="s">
+        <v>44</v>
+      </c>
+      <c r="N23">
+        <v>22</v>
+      </c>
+      <c r="O23" t="s">
+        <v>43</v>
+      </c>
+      <c r="P23" t="s">
+        <v>848</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>455</v>
+      </c>
+      <c r="R23" t="s">
+        <v>44</v>
+      </c>
+      <c r="S23">
+        <v>14</v>
+      </c>
+      <c r="T23" t="s">
+        <v>48</v>
+      </c>
+      <c r="U23" t="s">
+        <v>849</v>
+      </c>
+      <c r="V23">
+        <v>22</v>
+      </c>
+      <c r="W23" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="X23" t="s">
+        <v>431</v>
+      </c>
+      <c r="Y23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>481</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>850</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>851</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" t="s">
+        <v>853</v>
+      </c>
+      <c r="D24" t="s">
+        <v>277</v>
+      </c>
+      <c r="E24" t="s">
+        <v>246</v>
+      </c>
+      <c r="F24" t="s">
+        <v>247</v>
+      </c>
+      <c r="G24" t="s">
+        <v>72</v>
+      </c>
+      <c r="H24" t="s">
+        <v>256</v>
+      </c>
+      <c r="I24" t="s">
+        <v>272</v>
+      </c>
+      <c r="J24" t="s">
+        <v>706</v>
+      </c>
+      <c r="K24" t="s">
+        <v>707</v>
+      </c>
+      <c r="L24" t="s">
+        <v>43</v>
+      </c>
+      <c r="M24" t="s">
+        <v>44</v>
+      </c>
+      <c r="N24">
+        <v>7</v>
+      </c>
+      <c r="O24" t="s">
+        <v>43</v>
+      </c>
+      <c r="P24" t="s">
+        <v>854</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>455</v>
+      </c>
+      <c r="R24" t="s">
+        <v>44</v>
+      </c>
+      <c r="S24">
+        <v>6</v>
+      </c>
+      <c r="T24" t="s">
+        <v>48</v>
+      </c>
+      <c r="U24" t="s">
+        <v>855</v>
+      </c>
+      <c r="V24">
+        <v>9</v>
+      </c>
+      <c r="W24" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="X24" t="s">
+        <v>856</v>
+      </c>
+      <c r="Y24" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>857</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>858</v>
+      </c>
+      <c r="AE24" t="s">
+        <v>859</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" t="s">
+        <v>861</v>
+      </c>
+      <c r="D25" t="s">
+        <v>287</v>
+      </c>
+      <c r="E25" t="s">
+        <v>246</v>
+      </c>
+      <c r="F25" t="s">
+        <v>247</v>
+      </c>
+      <c r="G25" t="s">
+        <v>72</v>
+      </c>
+      <c r="H25" t="s">
+        <v>272</v>
+      </c>
+      <c r="I25" t="s">
+        <v>249</v>
+      </c>
+      <c r="J25" t="s">
+        <v>706</v>
+      </c>
+      <c r="K25" t="s">
+        <v>707</v>
+      </c>
+      <c r="L25" t="s">
+        <v>43</v>
+      </c>
+      <c r="M25" t="s">
+        <v>44</v>
+      </c>
+      <c r="N25">
+        <v>4</v>
+      </c>
+      <c r="O25" t="s">
+        <v>43</v>
+      </c>
+      <c r="P25" t="s">
+        <v>862</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>455</v>
+      </c>
+      <c r="R25" t="s">
+        <v>44</v>
+      </c>
+      <c r="S25">
+        <v>3</v>
+      </c>
+      <c r="T25" t="s">
+        <v>48</v>
+      </c>
+      <c r="U25" t="s">
+        <v>863</v>
+      </c>
+      <c r="V25">
+        <v>3</v>
+      </c>
+      <c r="W25" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="X25" t="s">
+        <v>160</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>864</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>865</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>866</v>
+      </c>
+      <c r="AE25" t="s">
+        <v>867</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" t="s">
+        <v>869</v>
+      </c>
+      <c r="D26" t="s">
+        <v>297</v>
+      </c>
+      <c r="E26" t="s">
+        <v>298</v>
+      </c>
+      <c r="F26" t="s">
+        <v>299</v>
+      </c>
+      <c r="G26" t="s">
+        <v>72</v>
+      </c>
+      <c r="H26" t="s">
+        <v>300</v>
+      </c>
+      <c r="I26" t="s">
+        <v>301</v>
+      </c>
+      <c r="J26" t="s">
+        <v>706</v>
+      </c>
+      <c r="K26" t="s">
+        <v>707</v>
+      </c>
+      <c r="L26" t="s">
+        <v>870</v>
+      </c>
+      <c r="M26" t="s">
+        <v>44</v>
+      </c>
+      <c r="N26">
+        <v>26</v>
+      </c>
+      <c r="O26" t="s">
+        <v>45</v>
+      </c>
+      <c r="P26" t="s">
+        <v>871</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>304</v>
+      </c>
+      <c r="R26" t="s">
+        <v>44</v>
+      </c>
+      <c r="S26">
+        <v>9</v>
+      </c>
+      <c r="T26" t="s">
+        <v>48</v>
+      </c>
+      <c r="U26" t="s">
+        <v>872</v>
+      </c>
+      <c r="V26">
+        <v>21</v>
+      </c>
+      <c r="W26" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="X26" t="s">
+        <v>873</v>
+      </c>
+      <c r="Y26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>874</v>
+      </c>
+      <c r="AA26" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC26" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD26" t="s">
+        <v>875</v>
+      </c>
+      <c r="AE26" t="s">
+        <v>876</v>
+      </c>
+      <c r="AF26" t="s">
+        <v>877</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AF1"/>
+  <hyperlinks>
+    <hyperlink ref="AA2" r:id="rId1"/>
+    <hyperlink ref="AB2" r:id="rId2"/>
+    <hyperlink ref="AC2" r:id="rId3"/>
+    <hyperlink ref="AA3" r:id="rId4"/>
+    <hyperlink ref="AB3" r:id="rId5"/>
+    <hyperlink ref="AC3" r:id="rId6"/>
+    <hyperlink ref="AA4" r:id="rId7"/>
+    <hyperlink ref="AB4" r:id="rId8"/>
+    <hyperlink ref="AC4" r:id="rId9"/>
+    <hyperlink ref="AA5" r:id="rId10"/>
+    <hyperlink ref="AB5" r:id="rId11"/>
+    <hyperlink ref="AC5" r:id="rId12"/>
+    <hyperlink ref="AA6" r:id="rId13"/>
+    <hyperlink ref="AB6" r:id="rId14"/>
+    <hyperlink ref="AC6" r:id="rId15"/>
+    <hyperlink ref="AA7" r:id="rId16"/>
+    <hyperlink ref="AB7" r:id="rId17"/>
+    <hyperlink ref="AC7" r:id="rId18"/>
+    <hyperlink ref="AA8" r:id="rId19"/>
+    <hyperlink ref="AB8" r:id="rId20"/>
+    <hyperlink ref="AC8" r:id="rId21"/>
+    <hyperlink ref="AA9" r:id="rId22"/>
+    <hyperlink ref="AB9" r:id="rId23"/>
+    <hyperlink ref="AC9" r:id="rId24"/>
+    <hyperlink ref="AA10" r:id="rId25"/>
+    <hyperlink ref="AB10" r:id="rId26"/>
+    <hyperlink ref="AC10" r:id="rId27"/>
+    <hyperlink ref="AA11" r:id="rId28"/>
+    <hyperlink ref="AB11" r:id="rId29"/>
+    <hyperlink ref="AC11" r:id="rId30"/>
+    <hyperlink ref="AA12" r:id="rId31"/>
+    <hyperlink ref="AB12" r:id="rId32"/>
+    <hyperlink ref="AC12" r:id="rId33"/>
+    <hyperlink ref="AA13" r:id="rId34"/>
+    <hyperlink ref="AB13" r:id="rId35"/>
+    <hyperlink ref="AC13" r:id="rId36"/>
+    <hyperlink ref="AA14" r:id="rId37"/>
+    <hyperlink ref="AB14" r:id="rId38"/>
+    <hyperlink ref="AC14" r:id="rId39"/>
+    <hyperlink ref="AA15" r:id="rId40"/>
+    <hyperlink ref="AB15" r:id="rId41"/>
+    <hyperlink ref="AC15" r:id="rId42"/>
+    <hyperlink ref="AA16" r:id="rId43"/>
+    <hyperlink ref="AB16" r:id="rId44"/>
+    <hyperlink ref="AC16" r:id="rId45"/>
+    <hyperlink ref="AA17" r:id="rId46"/>
+    <hyperlink ref="AB17" r:id="rId47"/>
+    <hyperlink ref="AC17" r:id="rId48"/>
+    <hyperlink ref="AA18" r:id="rId49"/>
+    <hyperlink ref="AB18" r:id="rId50"/>
+    <hyperlink ref="AC18" r:id="rId51"/>
+    <hyperlink ref="AA19" r:id="rId52"/>
+    <hyperlink ref="AB19" r:id="rId53"/>
+    <hyperlink ref="AC19" r:id="rId54"/>
+    <hyperlink ref="AA20" r:id="rId55"/>
+    <hyperlink ref="AB20" r:id="rId56"/>
+    <hyperlink ref="AC20" r:id="rId57"/>
+    <hyperlink ref="AA21" r:id="rId58"/>
+    <hyperlink ref="AB21" r:id="rId59"/>
+    <hyperlink ref="AC21" r:id="rId60"/>
+    <hyperlink ref="AA22" r:id="rId61"/>
+    <hyperlink ref="AB22" r:id="rId62"/>
+    <hyperlink ref="AC22" r:id="rId63"/>
+    <hyperlink ref="AA23" r:id="rId64"/>
+    <hyperlink ref="AB23" r:id="rId65"/>
+    <hyperlink ref="AC23" r:id="rId66"/>
+    <hyperlink ref="AA24" r:id="rId67"/>
+    <hyperlink ref="AB24" r:id="rId68"/>
+    <hyperlink ref="AC24" r:id="rId69"/>
+    <hyperlink ref="AA25" r:id="rId70"/>
+    <hyperlink ref="AB25" r:id="rId71"/>
+    <hyperlink ref="AC25" r:id="rId72"/>
+    <hyperlink ref="AA26" r:id="rId73"/>
+    <hyperlink ref="AB26" r:id="rId74"/>
+    <hyperlink ref="AC26" r:id="rId75"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:BH26"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:60" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>3</v>
       </c>
@@ -10604,133 +13803,175 @@
         <v>8</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>705</v>
+        <v>878</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>706</v>
+        <v>879</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>707</v>
+        <v>880</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>708</v>
+        <v>881</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>709</v>
+        <v>882</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>710</v>
+        <v>883</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>711</v>
+        <v>884</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>712</v>
+        <v>885</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>713</v>
+        <v>886</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>714</v>
+        <v>887</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>715</v>
+        <v>888</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>716</v>
+        <v>889</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>717</v>
+        <v>890</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>718</v>
+        <v>891</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>719</v>
+        <v>892</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>720</v>
+        <v>893</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>721</v>
+        <v>894</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>722</v>
+        <v>895</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>723</v>
+        <v>896</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>724</v>
+        <v>897</v>
       </c>
       <c r="Y1" s="5" t="s">
-        <v>725</v>
+        <v>898</v>
       </c>
       <c r="Z1" s="5" t="s">
-        <v>726</v>
+        <v>899</v>
       </c>
       <c r="AA1" s="5" t="s">
-        <v>727</v>
+        <v>900</v>
       </c>
       <c r="AB1" s="5" t="s">
-        <v>728</v>
+        <v>901</v>
       </c>
       <c r="AC1" s="5" t="s">
-        <v>729</v>
+        <v>902</v>
       </c>
       <c r="AD1" s="5" t="s">
-        <v>730</v>
+        <v>903</v>
       </c>
       <c r="AE1" s="5" t="s">
-        <v>731</v>
+        <v>904</v>
       </c>
       <c r="AF1" s="5" t="s">
-        <v>732</v>
+        <v>905</v>
       </c>
       <c r="AG1" s="5" t="s">
-        <v>733</v>
+        <v>906</v>
       </c>
       <c r="AH1" s="5" t="s">
-        <v>734</v>
+        <v>907</v>
       </c>
       <c r="AI1" s="5" t="s">
-        <v>735</v>
+        <v>908</v>
       </c>
       <c r="AJ1" s="5" t="s">
-        <v>736</v>
+        <v>909</v>
       </c>
       <c r="AK1" s="5" t="s">
-        <v>737</v>
+        <v>910</v>
       </c>
       <c r="AL1" s="5" t="s">
-        <v>738</v>
+        <v>911</v>
       </c>
       <c r="AM1" s="5" t="s">
-        <v>739</v>
+        <v>912</v>
       </c>
       <c r="AN1" s="5" t="s">
-        <v>740</v>
+        <v>913</v>
       </c>
       <c r="AO1" s="5" t="s">
-        <v>741</v>
+        <v>914</v>
       </c>
       <c r="AP1" s="5" t="s">
-        <v>742</v>
+        <v>915</v>
       </c>
       <c r="AQ1" s="5" t="s">
-        <v>743</v>
+        <v>916</v>
       </c>
       <c r="AR1" s="5" t="s">
-        <v>744</v>
+        <v>917</v>
       </c>
       <c r="AS1" s="5" t="s">
-        <v>745</v>
+        <v>918</v>
       </c>
       <c r="AT1" s="5" t="s">
-        <v>746</v>
+        <v>919</v>
+      </c>
+      <c r="AU1" s="5" t="s">
+        <v>920</v>
+      </c>
+      <c r="AV1" s="5" t="s">
+        <v>921</v>
+      </c>
+      <c r="AW1" s="5" t="s">
+        <v>922</v>
+      </c>
+      <c r="AX1" s="5" t="s">
+        <v>923</v>
+      </c>
+      <c r="AY1" s="5" t="s">
+        <v>924</v>
+      </c>
+      <c r="AZ1" s="5" t="s">
+        <v>925</v>
+      </c>
+      <c r="BA1" s="5" t="s">
+        <v>926</v>
+      </c>
+      <c r="BB1" s="5" t="s">
+        <v>927</v>
+      </c>
+      <c r="BC1" s="5" t="s">
+        <v>928</v>
+      </c>
+      <c r="BD1" s="5" t="s">
+        <v>929</v>
+      </c>
+      <c r="BE1" s="5" t="s">
+        <v>930</v>
+      </c>
+      <c r="BF1" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="BG1" s="5" t="s">
+        <v>932</v>
+      </c>
+      <c r="BH1" s="5" t="s">
+        <v>933</v>
       </c>
     </row>
-    <row r="2" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>35</v>
       </c>
@@ -10869,8 +14110,50 @@
       <c r="AT2" t="s">
         <v>516</v>
       </c>
+      <c r="AU2" t="s">
+        <v>705</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX2">
+        <v>50</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>708</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>47</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC2">
+        <v>28</v>
+      </c>
+      <c r="BD2" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>709</v>
+      </c>
+      <c r="BF2">
+        <v>53</v>
+      </c>
+      <c r="BG2" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="3" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -11009,8 +14292,50 @@
       <c r="AT3" t="s">
         <v>184</v>
       </c>
+      <c r="AU3" t="s">
+        <v>713</v>
+      </c>
+      <c r="AV3" t="s">
+        <v>61</v>
+      </c>
+      <c r="AW3" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX3">
+        <v>51</v>
+      </c>
+      <c r="AY3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>714</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>47</v>
+      </c>
+      <c r="BB3" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC3">
+        <v>29</v>
+      </c>
+      <c r="BD3" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE3" t="s">
+        <v>715</v>
+      </c>
+      <c r="BF3">
+        <v>65</v>
+      </c>
+      <c r="BG3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH3" t="s">
+        <v>717</v>
+      </c>
     </row>
-    <row r="4" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -11149,8 +14474,50 @@
       <c r="AT4" t="s">
         <v>533</v>
       </c>
+      <c r="AU4" t="s">
+        <v>721</v>
+      </c>
+      <c r="AV4" t="s">
+        <v>336</v>
+      </c>
+      <c r="AW4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX4">
+        <v>12</v>
+      </c>
+      <c r="AY4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ4" t="s">
+        <v>722</v>
+      </c>
+      <c r="BA4" t="s">
+        <v>47</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC4">
+        <v>8</v>
+      </c>
+      <c r="BD4" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE4" t="s">
+        <v>723</v>
+      </c>
+      <c r="BF4">
+        <v>17</v>
+      </c>
+      <c r="BG4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH4" t="s">
+        <v>725</v>
+      </c>
     </row>
-    <row r="5" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>86</v>
       </c>
@@ -11289,8 +14656,50 @@
       <c r="AT5" t="s">
         <v>206</v>
       </c>
+      <c r="AU5" t="s">
+        <v>729</v>
+      </c>
+      <c r="AV5" t="s">
+        <v>87</v>
+      </c>
+      <c r="AW5" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX5">
+        <v>18</v>
+      </c>
+      <c r="AY5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ5" t="s">
+        <v>730</v>
+      </c>
+      <c r="BA5" t="s">
+        <v>47</v>
+      </c>
+      <c r="BB5" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC5">
+        <v>11</v>
+      </c>
+      <c r="BD5" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE5" t="s">
+        <v>731</v>
+      </c>
+      <c r="BF5">
+        <v>33</v>
+      </c>
+      <c r="BG5" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH5" t="s">
+        <v>92</v>
+      </c>
     </row>
-    <row r="6" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>97</v>
       </c>
@@ -11429,8 +14838,50 @@
       <c r="AT6" t="s">
         <v>92</v>
       </c>
+      <c r="AU6" t="s">
+        <v>735</v>
+      </c>
+      <c r="AV6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW6" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX6">
+        <v>18</v>
+      </c>
+      <c r="AY6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ6" t="s">
+        <v>736</v>
+      </c>
+      <c r="BA6" t="s">
+        <v>47</v>
+      </c>
+      <c r="BB6" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC6">
+        <v>11</v>
+      </c>
+      <c r="BD6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE6" t="s">
+        <v>737</v>
+      </c>
+      <c r="BF6">
+        <v>22</v>
+      </c>
+      <c r="BG6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH6" t="s">
+        <v>92</v>
+      </c>
     </row>
-    <row r="7" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>106</v>
       </c>
@@ -11569,8 +15020,50 @@
       <c r="AT7" t="s">
         <v>554</v>
       </c>
+      <c r="AU7" t="s">
+        <v>741</v>
+      </c>
+      <c r="AV7" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX7">
+        <v>24</v>
+      </c>
+      <c r="AY7" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ7" t="s">
+        <v>742</v>
+      </c>
+      <c r="BA7" t="s">
+        <v>47</v>
+      </c>
+      <c r="BB7" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC7">
+        <v>12</v>
+      </c>
+      <c r="BD7" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE7" t="s">
+        <v>743</v>
+      </c>
+      <c r="BF7">
+        <v>26</v>
+      </c>
+      <c r="BG7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH7" t="s">
+        <v>111</v>
+      </c>
     </row>
-    <row r="8" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>116</v>
       </c>
@@ -11709,8 +15202,50 @@
       <c r="AT8" t="s">
         <v>562</v>
       </c>
+      <c r="AU8" t="s">
+        <v>747</v>
+      </c>
+      <c r="AV8" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW8" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX8">
+        <v>27</v>
+      </c>
+      <c r="AY8" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ8" t="s">
+        <v>748</v>
+      </c>
+      <c r="BA8" t="s">
+        <v>47</v>
+      </c>
+      <c r="BB8" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC8">
+        <v>18</v>
+      </c>
+      <c r="BD8" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE8" t="s">
+        <v>749</v>
+      </c>
+      <c r="BF8">
+        <v>37</v>
+      </c>
+      <c r="BG8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH8" t="s">
+        <v>725</v>
+      </c>
     </row>
-    <row r="9" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>129</v>
       </c>
@@ -11849,8 +15384,50 @@
       <c r="AT9" t="s">
         <v>570</v>
       </c>
+      <c r="AU9" t="s">
+        <v>753</v>
+      </c>
+      <c r="AV9" t="s">
+        <v>61</v>
+      </c>
+      <c r="AW9" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX9">
+        <v>22</v>
+      </c>
+      <c r="AY9" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ9" t="s">
+        <v>754</v>
+      </c>
+      <c r="BA9" t="s">
+        <v>47</v>
+      </c>
+      <c r="BB9" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC9">
+        <v>15</v>
+      </c>
+      <c r="BD9" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE9" t="s">
+        <v>755</v>
+      </c>
+      <c r="BF9">
+        <v>33</v>
+      </c>
+      <c r="BG9" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH9" t="s">
+        <v>134</v>
+      </c>
     </row>
-    <row r="10" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>139</v>
       </c>
@@ -11989,8 +15566,50 @@
       <c r="AT10" t="s">
         <v>579</v>
       </c>
+      <c r="AU10" t="s">
+        <v>759</v>
+      </c>
+      <c r="AV10" t="s">
+        <v>336</v>
+      </c>
+      <c r="AW10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX10">
+        <v>30</v>
+      </c>
+      <c r="AY10" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ10" t="s">
+        <v>760</v>
+      </c>
+      <c r="BA10" t="s">
+        <v>47</v>
+      </c>
+      <c r="BB10" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC10">
+        <v>16</v>
+      </c>
+      <c r="BD10" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE10" t="s">
+        <v>761</v>
+      </c>
+      <c r="BF10">
+        <v>47</v>
+      </c>
+      <c r="BG10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH10" t="s">
+        <v>764</v>
+      </c>
     </row>
-    <row r="11" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>151</v>
       </c>
@@ -12129,8 +15748,50 @@
       <c r="AT11" t="s">
         <v>588</v>
       </c>
+      <c r="AU11" t="s">
+        <v>768</v>
+      </c>
+      <c r="AV11" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW11" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX11">
+        <v>40</v>
+      </c>
+      <c r="AY11" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ11" t="s">
+        <v>769</v>
+      </c>
+      <c r="BA11" t="s">
+        <v>157</v>
+      </c>
+      <c r="BB11" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC11">
+        <v>30</v>
+      </c>
+      <c r="BD11" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE11" t="s">
+        <v>770</v>
+      </c>
+      <c r="BF11">
+        <v>63</v>
+      </c>
+      <c r="BG11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH11" t="s">
+        <v>377</v>
+      </c>
     </row>
-    <row r="12" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>167</v>
       </c>
@@ -12269,8 +15930,50 @@
       <c r="AT12" t="s">
         <v>596</v>
       </c>
+      <c r="AU12" t="s">
+        <v>774</v>
+      </c>
+      <c r="AV12" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW12" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX12">
+        <v>25</v>
+      </c>
+      <c r="AY12" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ12" t="s">
+        <v>775</v>
+      </c>
+      <c r="BA12" t="s">
+        <v>157</v>
+      </c>
+      <c r="BB12" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC12">
+        <v>21</v>
+      </c>
+      <c r="BD12" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE12" t="s">
+        <v>776</v>
+      </c>
+      <c r="BF12">
+        <v>31</v>
+      </c>
+      <c r="BG12" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH12" t="s">
+        <v>596</v>
+      </c>
     </row>
-    <row r="13" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>178</v>
       </c>
@@ -12409,8 +16112,50 @@
       <c r="AT13" t="s">
         <v>604</v>
       </c>
+      <c r="AU13" t="s">
+        <v>780</v>
+      </c>
+      <c r="AV13" t="s">
+        <v>180</v>
+      </c>
+      <c r="AW13" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX13">
+        <v>17</v>
+      </c>
+      <c r="AY13" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ13" t="s">
+        <v>781</v>
+      </c>
+      <c r="BA13" t="s">
+        <v>157</v>
+      </c>
+      <c r="BB13" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC13">
+        <v>11</v>
+      </c>
+      <c r="BD13" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE13" t="s">
+        <v>782</v>
+      </c>
+      <c r="BF13">
+        <v>37</v>
+      </c>
+      <c r="BG13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH13" t="s">
+        <v>604</v>
+      </c>
     </row>
-    <row r="14" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>189</v>
       </c>
@@ -12549,8 +16294,50 @@
       <c r="AT14" t="s">
         <v>612</v>
       </c>
+      <c r="AU14" t="s">
+        <v>786</v>
+      </c>
+      <c r="AV14" t="s">
+        <v>787</v>
+      </c>
+      <c r="AW14" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX14">
+        <v>25</v>
+      </c>
+      <c r="AY14" t="s">
+        <v>45</v>
+      </c>
+      <c r="AZ14" t="s">
+        <v>788</v>
+      </c>
+      <c r="BA14" t="s">
+        <v>157</v>
+      </c>
+      <c r="BB14" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC14">
+        <v>18</v>
+      </c>
+      <c r="BD14" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE14" t="s">
+        <v>789</v>
+      </c>
+      <c r="BF14">
+        <v>24</v>
+      </c>
+      <c r="BG14" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH14" t="s">
+        <v>791</v>
+      </c>
     </row>
-    <row r="15" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>201</v>
       </c>
@@ -12689,8 +16476,50 @@
       <c r="AT15" t="s">
         <v>622</v>
       </c>
+      <c r="AU15" t="s">
+        <v>795</v>
+      </c>
+      <c r="AV15" t="s">
+        <v>617</v>
+      </c>
+      <c r="AW15" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX15">
+        <v>23</v>
+      </c>
+      <c r="AY15" t="s">
+        <v>141</v>
+      </c>
+      <c r="AZ15" t="s">
+        <v>796</v>
+      </c>
+      <c r="BA15" t="s">
+        <v>157</v>
+      </c>
+      <c r="BB15" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC15">
+        <v>12</v>
+      </c>
+      <c r="BD15" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE15" t="s">
+        <v>797</v>
+      </c>
+      <c r="BF15">
+        <v>45</v>
+      </c>
+      <c r="BG15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH15" t="s">
+        <v>622</v>
+      </c>
     </row>
-    <row r="16" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>211</v>
       </c>
@@ -12829,8 +16658,50 @@
       <c r="AT16" t="s">
         <v>421</v>
       </c>
+      <c r="AU16" t="s">
+        <v>801</v>
+      </c>
+      <c r="AV16" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW16" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX16">
+        <v>34</v>
+      </c>
+      <c r="AY16" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ16" t="s">
+        <v>802</v>
+      </c>
+      <c r="BA16" t="s">
+        <v>157</v>
+      </c>
+      <c r="BB16" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC16">
+        <v>25</v>
+      </c>
+      <c r="BD16" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE16" t="s">
+        <v>803</v>
+      </c>
+      <c r="BF16">
+        <v>49</v>
+      </c>
+      <c r="BG16" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH16" t="s">
+        <v>421</v>
+      </c>
     </row>
-    <row r="17" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>221</v>
       </c>
@@ -12969,8 +16840,50 @@
       <c r="AT17" t="s">
         <v>636</v>
       </c>
+      <c r="AU17" t="s">
+        <v>807</v>
+      </c>
+      <c r="AV17" t="s">
+        <v>426</v>
+      </c>
+      <c r="AW17" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX17">
+        <v>36</v>
+      </c>
+      <c r="AY17" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ17" t="s">
+        <v>808</v>
+      </c>
+      <c r="BA17" t="s">
+        <v>428</v>
+      </c>
+      <c r="BB17" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC17">
+        <v>28</v>
+      </c>
+      <c r="BD17" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE17" t="s">
+        <v>634</v>
+      </c>
+      <c r="BF17">
+        <v>42</v>
+      </c>
+      <c r="BG17" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH17" t="s">
+        <v>809</v>
+      </c>
     </row>
-    <row r="18" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>231</v>
       </c>
@@ -13109,8 +17022,50 @@
       <c r="AT18" t="s">
         <v>644</v>
       </c>
+      <c r="AU18" t="s">
+        <v>813</v>
+      </c>
+      <c r="AV18" t="s">
+        <v>814</v>
+      </c>
+      <c r="AW18" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX18">
+        <v>16</v>
+      </c>
+      <c r="AY18" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ18" t="s">
+        <v>815</v>
+      </c>
+      <c r="BA18" t="s">
+        <v>428</v>
+      </c>
+      <c r="BB18" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC18">
+        <v>17</v>
+      </c>
+      <c r="BD18" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE18" t="s">
+        <v>816</v>
+      </c>
+      <c r="BF18">
+        <v>27</v>
+      </c>
+      <c r="BG18" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="BH18" t="s">
+        <v>819</v>
+      </c>
     </row>
-    <row r="19" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>238</v>
       </c>
@@ -13249,8 +17204,50 @@
       <c r="AT19" t="s">
         <v>654</v>
       </c>
+      <c r="AU19" t="s">
+        <v>823</v>
+      </c>
+      <c r="AV19" t="s">
+        <v>444</v>
+      </c>
+      <c r="AW19" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX19">
+        <v>47</v>
+      </c>
+      <c r="AY19" t="s">
+        <v>119</v>
+      </c>
+      <c r="AZ19" t="s">
+        <v>824</v>
+      </c>
+      <c r="BA19" t="s">
+        <v>428</v>
+      </c>
+      <c r="BB19" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC19">
+        <v>23</v>
+      </c>
+      <c r="BD19" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE19" t="s">
+        <v>651</v>
+      </c>
+      <c r="BF19">
+        <v>40</v>
+      </c>
+      <c r="BG19" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH19" t="s">
+        <v>825</v>
+      </c>
     </row>
-    <row r="20" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>245</v>
       </c>
@@ -13389,8 +17386,50 @@
       <c r="AT20" t="s">
         <v>458</v>
       </c>
+      <c r="AU20" t="s">
+        <v>829</v>
+      </c>
+      <c r="AV20" t="s">
+        <v>250</v>
+      </c>
+      <c r="AW20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX20">
+        <v>26</v>
+      </c>
+      <c r="AY20" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ20" t="s">
+        <v>830</v>
+      </c>
+      <c r="BA20" t="s">
+        <v>455</v>
+      </c>
+      <c r="BB20" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC20">
+        <v>17</v>
+      </c>
+      <c r="BD20" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE20" t="s">
+        <v>831</v>
+      </c>
+      <c r="BF20">
+        <v>25</v>
+      </c>
+      <c r="BG20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH20" t="s">
+        <v>458</v>
+      </c>
     </row>
-    <row r="21" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>255</v>
       </c>
@@ -13529,8 +17568,50 @@
       <c r="AT21" t="s">
         <v>668</v>
       </c>
+      <c r="AU21" t="s">
+        <v>835</v>
+      </c>
+      <c r="AV21" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW21" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX21">
+        <v>12</v>
+      </c>
+      <c r="AY21" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ21" t="s">
+        <v>836</v>
+      </c>
+      <c r="BA21" t="s">
+        <v>455</v>
+      </c>
+      <c r="BB21" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC21">
+        <v>9</v>
+      </c>
+      <c r="BD21" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE21" t="s">
+        <v>837</v>
+      </c>
+      <c r="BF21">
+        <v>11</v>
+      </c>
+      <c r="BG21" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH21" t="s">
+        <v>377</v>
+      </c>
     </row>
-    <row r="22" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>261</v>
       </c>
@@ -13669,8 +17750,50 @@
       <c r="AT22" t="s">
         <v>674</v>
       </c>
+      <c r="AU22" t="s">
+        <v>841</v>
+      </c>
+      <c r="AV22" t="s">
+        <v>250</v>
+      </c>
+      <c r="AW22" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX22">
+        <v>14</v>
+      </c>
+      <c r="AY22" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ22" t="s">
+        <v>842</v>
+      </c>
+      <c r="BA22" t="s">
+        <v>455</v>
+      </c>
+      <c r="BB22" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC22">
+        <v>8</v>
+      </c>
+      <c r="BD22" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE22" t="s">
+        <v>843</v>
+      </c>
+      <c r="BF22">
+        <v>13</v>
+      </c>
+      <c r="BG22" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH22" t="s">
+        <v>474</v>
+      </c>
     </row>
-    <row r="23" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>271</v>
       </c>
@@ -13809,8 +17932,50 @@
       <c r="AT23" t="s">
         <v>481</v>
       </c>
+      <c r="AU23" t="s">
+        <v>847</v>
+      </c>
+      <c r="AV23" t="s">
+        <v>250</v>
+      </c>
+      <c r="AW23" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX23">
+        <v>22</v>
+      </c>
+      <c r="AY23" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ23" t="s">
+        <v>848</v>
+      </c>
+      <c r="BA23" t="s">
+        <v>455</v>
+      </c>
+      <c r="BB23" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC23">
+        <v>14</v>
+      </c>
+      <c r="BD23" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE23" t="s">
+        <v>849</v>
+      </c>
+      <c r="BF23">
+        <v>22</v>
+      </c>
+      <c r="BG23" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH23" t="s">
+        <v>481</v>
+      </c>
     </row>
-    <row r="24" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>277</v>
       </c>
@@ -13949,8 +18114,50 @@
       <c r="AT24" t="s">
         <v>686</v>
       </c>
+      <c r="AU24" t="s">
+        <v>853</v>
+      </c>
+      <c r="AV24" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW24" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX24">
+        <v>7</v>
+      </c>
+      <c r="AY24" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ24" t="s">
+        <v>854</v>
+      </c>
+      <c r="BA24" t="s">
+        <v>455</v>
+      </c>
+      <c r="BB24" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC24">
+        <v>6</v>
+      </c>
+      <c r="BD24" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE24" t="s">
+        <v>855</v>
+      </c>
+      <c r="BF24">
+        <v>9</v>
+      </c>
+      <c r="BG24" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH24" t="s">
+        <v>857</v>
+      </c>
     </row>
-    <row r="25" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>287</v>
       </c>
@@ -14089,8 +18296,50 @@
       <c r="AT25" t="s">
         <v>292</v>
       </c>
+      <c r="AU25" t="s">
+        <v>861</v>
+      </c>
+      <c r="AV25" t="s">
+        <v>43</v>
+      </c>
+      <c r="AW25" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX25">
+        <v>4</v>
+      </c>
+      <c r="AY25" t="s">
+        <v>43</v>
+      </c>
+      <c r="AZ25" t="s">
+        <v>862</v>
+      </c>
+      <c r="BA25" t="s">
+        <v>455</v>
+      </c>
+      <c r="BB25" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC25">
+        <v>3</v>
+      </c>
+      <c r="BD25" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE25" t="s">
+        <v>863</v>
+      </c>
+      <c r="BF25">
+        <v>3</v>
+      </c>
+      <c r="BG25" t="s">
+        <v>864</v>
+      </c>
+      <c r="BH25" t="s">
+        <v>865</v>
+      </c>
     </row>
-    <row r="26" spans="1:46" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>297</v>
       </c>
@@ -14229,9 +18478,51 @@
       <c r="AT26" t="s">
         <v>701</v>
       </c>
+      <c r="AU26" t="s">
+        <v>869</v>
+      </c>
+      <c r="AV26" t="s">
+        <v>870</v>
+      </c>
+      <c r="AW26" t="s">
+        <v>44</v>
+      </c>
+      <c r="AX26">
+        <v>26</v>
+      </c>
+      <c r="AY26" t="s">
+        <v>45</v>
+      </c>
+      <c r="AZ26" t="s">
+        <v>871</v>
+      </c>
+      <c r="BA26" t="s">
+        <v>304</v>
+      </c>
+      <c r="BB26" t="s">
+        <v>44</v>
+      </c>
+      <c r="BC26">
+        <v>9</v>
+      </c>
+      <c r="BD26" t="s">
+        <v>48</v>
+      </c>
+      <c r="BE26" t="s">
+        <v>872</v>
+      </c>
+      <c r="BF26">
+        <v>21</v>
+      </c>
+      <c r="BG26" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="BH26" t="s">
+        <v>874</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AT1"/>
+  <autoFilter ref="A1:BH1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>